<commit_message>
🔒 [FULL] Daily chip data 2026-07-01 22:53
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨+26/5d-190)&quot;;-0&quot; 億 (昨+26/5d-190)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +70億 &quot;&quot;(昨12/5d12)&quot;"/>
-    <numFmt numFmtId="167" formatCode="0.0%&quot; 市-722億 &quot;&quot;(昨20/5d18)&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.0%&quot; 市-720億 &quot;&quot;(昨20/5d18)&quot;"/>
     <numFmt numFmtId="168" formatCode="&quot;📅 明日預測 ↕ 中性 &quot;0.0&quot;% 信心 — P/C Ratio 主推 — 3 檔焦點&quot;"/>
     <numFmt numFmtId="169" formatCode="0.00%;[Color10]-0.00%"/>
     <numFmt numFmtId="170" formatCode="0.0%"/>
@@ -1818,7 +1818,7 @@
         <v>13</v>
       </c>
       <c r="F19" s="16" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G19" s="17" t="inlineStr">
         <is>
@@ -1826,7 +1826,7 @@
         </is>
       </c>
       <c r="H19" s="18" t="n">
-        <v>13571</v>
+        <v>14365</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
         <v>10</v>
       </c>
       <c r="N19" s="18" t="n">
-        <v>52338</v>
+        <v>53132</v>
       </c>
     </row>
     <row r="20">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="J22" s="19" t="n">
-        <v>6490</v>
+        <v>7158</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -2001,7 +2001,7 @@
         <v>9</v>
       </c>
       <c r="N22" s="18" t="n">
-        <v>30505</v>
+        <v>31173</v>
       </c>
     </row>
     <row r="23">
@@ -2022,7 +2022,7 @@
         <v>12</v>
       </c>
       <c r="F23" s="16" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G23" s="17" t="inlineStr">
         <is>
@@ -2042,17 +2042,17 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>張濬安</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="L23" s="19" t="n">
-        <v>1726</v>
+        <v>2461</v>
       </c>
       <c r="M23" s="20" t="n">
         <v>9</v>
       </c>
       <c r="N23" s="18" t="n">
-        <v>21324</v>
+        <v>22879</v>
       </c>
     </row>
     <row r="24">
@@ -2112,27 +2112,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2357</t>
+          <t>6770</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>📌 華碩</t>
+          <t>📌 力積電</t>
         </is>
       </c>
       <c r="E25" s="15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
-          <t>竹科主力分點</t>
+          <t>張濬安</t>
         </is>
       </c>
       <c r="H25" s="18" t="n">
-        <v>6021</v>
+        <v>4403</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -2140,7 +2140,7 @@
         </is>
       </c>
       <c r="J25" s="19" t="n">
-        <v>2551</v>
+        <v>2523</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -2148,13 +2148,13 @@
         </is>
       </c>
       <c r="L25" s="19" t="n">
-        <v>2204</v>
+        <v>2250</v>
       </c>
       <c r="M25" s="20" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N25" s="18" t="n">
-        <v>16403</v>
+        <v>17167</v>
       </c>
     </row>
     <row r="26">
@@ -2163,27 +2163,27 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>6770</t>
+          <t>2357</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>📌 力積電</t>
+          <t>📌 華碩</t>
         </is>
       </c>
       <c r="E26" s="15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F26" s="16" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
-          <t>張濬安</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="H26" s="18" t="n">
-        <v>4403</v>
+        <v>6021</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -2191,7 +2191,7 @@
         </is>
       </c>
       <c r="J26" s="19" t="n">
-        <v>2523</v>
+        <v>2551</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -2199,13 +2199,13 @@
         </is>
       </c>
       <c r="L26" s="19" t="n">
-        <v>2250</v>
+        <v>2204</v>
       </c>
       <c r="M26" s="20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N26" s="18" t="n">
-        <v>16268</v>
+        <v>16403</v>
       </c>
     </row>
     <row r="27">
@@ -2230,19 +2230,19 @@
       </c>
       <c r="G27" s="17" t="inlineStr">
         <is>
+          <t>陳族元</t>
+        </is>
+      </c>
+      <c r="H27" s="18" t="n">
+        <v>1310</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
           <t>強森</t>
         </is>
       </c>
-      <c r="H27" s="18" t="n">
+      <c r="J27" s="19" t="n">
         <v>1004</v>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>陳族元</t>
-        </is>
-      </c>
-      <c r="J27" s="19" t="n">
-        <v>858</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -2256,7 +2256,7 @@
         <v>10</v>
       </c>
       <c r="N27" s="18" t="n">
-        <v>5062</v>
+        <v>5513</v>
       </c>
     </row>
     <row r="28">
@@ -2274,10 +2274,10 @@
         </is>
       </c>
       <c r="E28" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F28" s="16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
@@ -2304,10 +2304,10 @@
         <v>302</v>
       </c>
       <c r="M28" s="20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N28" s="18" t="n">
-        <v>3056</v>
+        <v>3124</v>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="G31" s="196" t="n">
-        <v>-69.29268999999999</v>
+        <v>-67.94410000000001</v>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1">
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="G32" s="198" t="n">
-        <v>0.2066133272140842</v>
+        <v>0.206919138606294</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
@@ -2429,11 +2429,11 @@
         </is>
       </c>
       <c r="D38" s="33" t="n">
-        <v>2833870</v>
+        <v>2850916</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>38.9%</t>
+          <t>39.1%</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>25.4%</t>
+          <t>25.3%</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2631,12 +2631,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 11 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 12 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>11 檔</t>
+          <t>12 檔</t>
         </is>
       </c>
     </row>
@@ -3173,7 +3173,7 @@
         </is>
       </c>
       <c r="C72" s="33" t="n">
-        <v>2776908</v>
+        <v>2794292</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3200,7 +3200,7 @@
         <v>198077</v>
       </c>
       <c r="J72" s="202" t="n">
-        <v>0.2875925512129766</v>
+        <v>0.285803447077483</v>
       </c>
     </row>
     <row r="73">
@@ -3650,7 +3650,7 @@
     <row r="86" ht="22" customHeight="1">
       <c r="B86" s="59" t="inlineStr">
         <is>
-          <t>▍ G. 注意股 (資料日 20260630)</t>
+          <t>▍ G. 注意股 (資料日 20260701)</t>
         </is>
       </c>
     </row>
@@ -3696,7 +3696,7 @@
         <v>1</v>
       </c>
       <c r="E88" t="n">
-        <v>13.2</v>
+        <v>14.9</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -3719,7 +3719,7 @@
         <v>1</v>
       </c>
       <c r="E89" s="41" t="n">
-        <v>27.35</v>
+        <v>30.05</v>
       </c>
       <c r="F89" s="41" t="inlineStr">
         <is>
@@ -3742,7 +3742,7 @@
         <v>1</v>
       </c>
       <c r="E90" t="n">
-        <v>8.960000000000001</v>
+        <v>9.35</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -3753,276 +3753,276 @@
     <row r="91">
       <c r="B91" s="41" t="inlineStr">
         <is>
-          <t>1718</t>
+          <t>1447</t>
         </is>
       </c>
       <c r="C91" s="41" t="inlineStr">
         <is>
-          <t>中纖</t>
+          <t>力鵬</t>
         </is>
       </c>
       <c r="D91" s="41" t="n">
         <v>1</v>
       </c>
       <c r="E91" s="41" t="n">
-        <v>13.45</v>
+        <v>8.27</v>
       </c>
       <c r="F91" s="41" t="inlineStr">
         <is>
-          <t>56.04</t>
+          <t>-----</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="B92" t="inlineStr">
         <is>
-          <t>2233</t>
+          <t>1617</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>宇隆</t>
+          <t>榮星</t>
         </is>
       </c>
       <c r="D92" t="n">
         <v>1</v>
       </c>
       <c r="E92" t="n">
-        <v>212</v>
+        <v>22.85</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>33.81</t>
+          <t>25.97</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="B93" s="41" t="inlineStr">
         <is>
-          <t>2303</t>
+          <t>1710</t>
         </is>
       </c>
       <c r="C93" s="41" t="inlineStr">
         <is>
-          <t>聯電</t>
+          <t>東聯</t>
         </is>
       </c>
       <c r="D93" s="41" t="n">
         <v>1</v>
       </c>
       <c r="E93" s="41" t="n">
-        <v>164.5</v>
+        <v>18.4</v>
       </c>
       <c r="F93" s="41" t="inlineStr">
         <is>
-          <t>41.33</t>
+          <t>-----</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>2375</t>
+          <t>1718</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>凱美</t>
+          <t>中纖</t>
         </is>
       </c>
       <c r="D94" t="n">
         <v>1</v>
       </c>
       <c r="E94" t="n">
-        <v>211.5</v>
+        <v>12.4</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>64.29</t>
+          <t>51.67</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="B95" s="41" t="inlineStr">
         <is>
-          <t>2415</t>
+          <t>2243</t>
         </is>
       </c>
       <c r="C95" s="41" t="inlineStr">
         <is>
-          <t>錩新</t>
+          <t>宏旭-KY</t>
         </is>
       </c>
       <c r="D95" s="41" t="n">
         <v>1</v>
       </c>
       <c r="E95" s="41" t="n">
-        <v>37.5</v>
+        <v>62</v>
       </c>
       <c r="F95" s="41" t="inlineStr">
         <is>
-          <t>19.53</t>
+          <t>24.90</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
-          <t>2472</t>
+          <t>2303</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>立隆電</t>
+          <t>聯電</t>
         </is>
       </c>
       <c r="D96" t="n">
         <v>1</v>
       </c>
       <c r="E96" t="n">
-        <v>453.5</v>
+        <v>169</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>52.43</t>
+          <t>42.46</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="B97" s="41" t="inlineStr">
         <is>
-          <t>2483</t>
+          <t>2345</t>
         </is>
       </c>
       <c r="C97" s="41" t="inlineStr">
         <is>
-          <t>百容</t>
+          <t>智邦</t>
         </is>
       </c>
       <c r="D97" s="41" t="n">
         <v>1</v>
       </c>
       <c r="E97" s="41" t="n">
-        <v>57.1</v>
+        <v>2660</v>
       </c>
       <c r="F97" s="41" t="inlineStr">
         <is>
-          <t>62.07</t>
+          <t>50.30</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="B98" t="inlineStr">
         <is>
-          <t>2906</t>
+          <t>2363</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>高林</t>
+          <t>矽統</t>
         </is>
       </c>
       <c r="D98" t="n">
         <v>1</v>
       </c>
       <c r="E98" t="n">
-        <v>14.55</v>
+        <v>73.5</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>32.33</t>
+          <t>43.24</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="B99" s="41" t="inlineStr">
         <is>
-          <t>3016</t>
+          <t>2375</t>
         </is>
       </c>
       <c r="C99" s="41" t="inlineStr">
         <is>
-          <t>嘉晶</t>
+          <t>凱美</t>
         </is>
       </c>
       <c r="D99" s="41" t="n">
         <v>1</v>
       </c>
       <c r="E99" s="41" t="n">
-        <v>133.5</v>
+        <v>232.5</v>
       </c>
       <c r="F99" s="41" t="inlineStr">
         <is>
-          <t>325.61</t>
+          <t>70.67</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="B100" t="inlineStr">
         <is>
-          <t>3023</t>
+          <t>2406</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>信邦</t>
+          <t>國碩</t>
         </is>
       </c>
       <c r="D100" t="n">
         <v>1</v>
       </c>
       <c r="E100" t="n">
-        <v>328.5</v>
+        <v>40.2</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>25.72</t>
+          <t>-----</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" s="41" t="inlineStr">
         <is>
-          <t>3167</t>
+          <t>2484</t>
         </is>
       </c>
       <c r="C101" s="41" t="inlineStr">
         <is>
-          <t>大量</t>
+          <t>希華</t>
         </is>
       </c>
       <c r="D101" s="41" t="n">
         <v>1</v>
       </c>
       <c r="E101" s="41" t="n">
-        <v>842</v>
+        <v>79.8</v>
       </c>
       <c r="F101" s="41" t="inlineStr">
         <is>
-          <t>82.07</t>
+          <t>107.84</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>3189</t>
+          <t>3023</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>景碩</t>
+          <t>信邦</t>
         </is>
       </c>
       <c r="D102" t="n">
         <v>1</v>
       </c>
       <c r="E102" t="n">
-        <v>891</v>
+        <v>333</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>250.99</t>
+          <t>26.08</t>
         </is>
       </c>
     </row>
@@ -4386,7 +4386,7 @@
     <row r="122" ht="22" customHeight="1">
       <c r="B122" s="65" t="inlineStr">
         <is>
-          <t>▍ I. 未來 30 天除權息 (有效 260 檔, 已剔除過期)</t>
+          <t>▍ I. 未來 30 天除權息 (有效 306 檔, 已剔除過期)</t>
         </is>
       </c>
     </row>
@@ -5094,7 +5094,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="C29" s="70" t="inlineStr">
         <is>
-          <t>-69 億 淨買</t>
+          <t>-68 億 淨買</t>
         </is>
       </c>
     </row>
@@ -6097,7 +6097,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="B3" s="98" t="inlineStr">
         <is>
-          <t>大牌分析師 近 50/50 交易日出手 2419 次 (517 檔), 風格分布: 隔日沖近似 38% / 當沖 13% / 留倉 48%, 漲停命中 5% (其中 🔒鎖漲停 4%), 前 5 大集中 24%, 長線部位 58% (32 檔), ⚠️ 處置股部位 14% (40 檔), 📦 連續囤貨 28 檔 (最長 13 天 009816, 皆已停止)。 主軸: 高頻交易/持續進場/📦 連續囤貨。</t>
+          <t>大牌分析師 近 50/50 交易日出手 2419 次 (517 檔), 風格分布: 隔日沖近似 38% / 當沖 13% / 留倉 48%, 漲停命中 5% (其中 🔒鎖漲停 4%), 前 5 大集中 24%, 長線部位 58% (32 檔), ⚠️ 處置股部位 14% (48 檔), 📦 連續囤貨 28 檔 (最長 13 天 009816, 皆已停止)。 主軸: 高頻交易/持續進場/📦 連續囤貨。</t>
         </is>
       </c>
     </row>
@@ -13657,10 +13657,10 @@
         </is>
       </c>
       <c r="E189" s="129" t="n">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="F189" s="129" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G189" s="129" t="n">
         <v>11302</v>
@@ -13672,10 +13672,10 @@
         <v>9692</v>
       </c>
       <c r="J189" s="130" t="n">
-        <v>434.69</v>
+        <v>421.71</v>
       </c>
       <c r="K189" s="130" t="n">
-        <v>435.05</v>
+        <v>423.61</v>
       </c>
       <c r="L189" s="220">
         <f>F189*(K189-J189)</f>
@@ -13688,31 +13688,31 @@
       <c r="C190" s="131" t="n"/>
       <c r="D190" s="128" t="inlineStr">
         <is>
-          <t>智邦(2345)</t>
+          <t>聯電(2303)</t>
         </is>
       </c>
       <c r="E190" s="129" t="n">
-        <v>20</v>
+        <v>498</v>
       </c>
       <c r="F190" s="129" t="n">
-        <v>13</v>
+        <v>152</v>
       </c>
       <c r="G190" s="129" t="n">
-        <v>5230</v>
+        <v>8416</v>
       </c>
       <c r="H190" s="129" t="n">
-        <v>3343</v>
+        <v>2569</v>
       </c>
       <c r="I190" s="129" t="n">
-        <v>1887</v>
+        <v>5847</v>
       </c>
       <c r="J190" s="130" t="n">
-        <v>2615.15</v>
+        <v>169</v>
       </c>
       <c r="K190" s="130" t="n">
-        <v>2571.38</v>
-      </c>
-      <c r="L190" s="219">
+        <v>169</v>
+      </c>
+      <c r="L190" s="220">
         <f>F190*(K190-J190)</f>
         <v/>
       </c>
@@ -13723,29 +13723,29 @@
       <c r="C191" s="131" t="n"/>
       <c r="D191" s="128" t="inlineStr">
         <is>
-          <t>聯發科(2454)</t>
+          <t>智邦(2345)</t>
         </is>
       </c>
       <c r="E191" s="129" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F191" s="129" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G191" s="129" t="n">
-        <v>4985</v>
+        <v>5230</v>
       </c>
       <c r="H191" s="129" t="n">
-        <v>4384</v>
+        <v>3343</v>
       </c>
       <c r="I191" s="129" t="n">
-        <v>601</v>
+        <v>1887</v>
       </c>
       <c r="J191" s="130" t="n">
-        <v>4531.73</v>
+        <v>2615.15</v>
       </c>
       <c r="K191" s="130" t="n">
-        <v>4384.4</v>
+        <v>2571.38</v>
       </c>
       <c r="L191" s="219">
         <f>F191*(K191-J191)</f>
@@ -13758,29 +13758,29 @@
       <c r="C192" s="131" t="n"/>
       <c r="D192" s="128" t="inlineStr">
         <is>
-          <t>國巨*(2327)</t>
+          <t>聯發科(2454)</t>
         </is>
       </c>
       <c r="E192" s="129" t="n">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="F192" s="129" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="G192" s="129" t="n">
-        <v>4778</v>
+        <v>4985</v>
       </c>
       <c r="H192" s="129" t="n">
-        <v>2361</v>
+        <v>4384</v>
       </c>
       <c r="I192" s="129" t="n">
-        <v>2417</v>
+        <v>601</v>
       </c>
       <c r="J192" s="130" t="n">
-        <v>1137.57</v>
+        <v>4531.73</v>
       </c>
       <c r="K192" s="130" t="n">
-        <v>1124.14</v>
+        <v>4384.4</v>
       </c>
       <c r="L192" s="219">
         <f>F192*(K192-J192)</f>
@@ -13793,29 +13793,29 @@
       <c r="C193" s="131" t="n"/>
       <c r="D193" s="128" t="inlineStr">
         <is>
-          <t>景碩(3189)</t>
+          <t>國巨*(2327)</t>
         </is>
       </c>
       <c r="E193" s="129" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="F193" s="129" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G193" s="129" t="n">
-        <v>4152</v>
+        <v>4778</v>
       </c>
       <c r="H193" s="129" t="n">
-        <v>2110</v>
+        <v>2361</v>
       </c>
       <c r="I193" s="129" t="n">
-        <v>2042</v>
+        <v>2417</v>
       </c>
       <c r="J193" s="130" t="n">
-        <v>883.49</v>
+        <v>1137.57</v>
       </c>
       <c r="K193" s="130" t="n">
-        <v>879.12</v>
+        <v>1124.14</v>
       </c>
       <c r="L193" s="219">
         <f>F193*(K193-J193)</f>
@@ -13828,31 +13828,31 @@
       <c r="C194" s="131" t="n"/>
       <c r="D194" s="128" t="inlineStr">
         <is>
-          <t>群創(3481)</t>
+          <t>景碩(3189)</t>
         </is>
       </c>
       <c r="E194" s="129" t="n">
-        <v>538</v>
+        <v>47</v>
       </c>
       <c r="F194" s="129" t="n">
-        <v>461</v>
+        <v>24</v>
       </c>
       <c r="G194" s="129" t="n">
-        <v>3761</v>
+        <v>4152</v>
       </c>
       <c r="H194" s="129" t="n">
-        <v>3227</v>
+        <v>2110</v>
       </c>
       <c r="I194" s="129" t="n">
-        <v>534</v>
+        <v>2042</v>
       </c>
       <c r="J194" s="130" t="n">
-        <v>69.90000000000001</v>
+        <v>883.49</v>
       </c>
       <c r="K194" s="130" t="n">
-        <v>70</v>
-      </c>
-      <c r="L194" s="220">
+        <v>879.12</v>
+      </c>
+      <c r="L194" s="219">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -13863,29 +13863,29 @@
       <c r="C195" s="131" t="n"/>
       <c r="D195" s="128" t="inlineStr">
         <is>
-          <t>創見(2451)</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E195" s="129" t="n">
-        <v>146</v>
+        <v>486</v>
       </c>
       <c r="F195" s="129" t="n">
-        <v>8</v>
+        <v>259</v>
       </c>
       <c r="G195" s="129" t="n">
-        <v>3703</v>
+        <v>3761</v>
       </c>
       <c r="H195" s="129" t="n">
-        <v>205</v>
+        <v>3227</v>
       </c>
       <c r="I195" s="129" t="n">
-        <v>3498</v>
+        <v>534</v>
       </c>
       <c r="J195" s="130" t="n">
-        <v>253.63</v>
+        <v>77.38</v>
       </c>
       <c r="K195" s="130" t="n">
-        <v>256.5</v>
+        <v>124.59</v>
       </c>
       <c r="L195" s="220">
         <f>F195*(K195-J195)</f>
@@ -13898,31 +13898,31 @@
       <c r="C196" s="131" t="n"/>
       <c r="D196" s="128" t="inlineStr">
         <is>
-          <t>臻鼎-KY(4958)</t>
+          <t>創見(2451)</t>
         </is>
       </c>
       <c r="E196" s="129" t="n">
-        <v>53</v>
+        <v>148</v>
       </c>
       <c r="F196" s="129" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="G196" s="129" t="n">
-        <v>3188</v>
+        <v>3703</v>
       </c>
       <c r="H196" s="129" t="n">
-        <v>1481</v>
+        <v>205</v>
       </c>
       <c r="I196" s="129" t="n">
-        <v>1707</v>
+        <v>3498</v>
       </c>
       <c r="J196" s="130" t="n">
-        <v>601.51</v>
+        <v>250.2</v>
       </c>
       <c r="K196" s="130" t="n">
-        <v>592.28</v>
-      </c>
-      <c r="L196" s="219">
+        <v>256.5</v>
+      </c>
+      <c r="L196" s="220">
         <f>F196*(K196-J196)</f>
         <v/>
       </c>
@@ -13933,31 +13933,31 @@
       <c r="C197" s="131" t="n"/>
       <c r="D197" s="128" t="inlineStr">
         <is>
-          <t>友達(2409)</t>
+          <t>臻鼎-KY(4958)</t>
         </is>
       </c>
       <c r="E197" s="129" t="n">
-        <v>963</v>
+        <v>55</v>
       </c>
       <c r="F197" s="129" t="n">
-        <v>910</v>
+        <v>29</v>
       </c>
       <c r="G197" s="129" t="n">
-        <v>2952</v>
+        <v>3188</v>
       </c>
       <c r="H197" s="129" t="n">
-        <v>2789</v>
+        <v>1481</v>
       </c>
       <c r="I197" s="129" t="n">
-        <v>163</v>
+        <v>1707</v>
       </c>
       <c r="J197" s="130" t="n">
-        <v>30.65</v>
+        <v>579.64</v>
       </c>
       <c r="K197" s="130" t="n">
-        <v>30.65</v>
-      </c>
-      <c r="L197" s="220">
+        <v>510.59</v>
+      </c>
+      <c r="L197" s="219">
         <f>F197*(K197-J197)</f>
         <v/>
       </c>
@@ -13972,10 +13972,10 @@
         </is>
       </c>
       <c r="E198" s="129" t="n">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="F198" s="129" t="n">
-        <v>63</v>
+        <v>102</v>
       </c>
       <c r="G198" s="129" t="n">
         <v>2888</v>
@@ -13987,12 +13987,12 @@
         <v>1654</v>
       </c>
       <c r="J198" s="130" t="n">
-        <v>193.83</v>
+        <v>209.28</v>
       </c>
       <c r="K198" s="130" t="n">
-        <v>195.92</v>
-      </c>
-      <c r="L198" s="220">
+        <v>121.01</v>
+      </c>
+      <c r="L198" s="219">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-07-02 00:13
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="13">
+  <numFmts count="14">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨+26/5d-190)&quot;;-0&quot; 億 (昨+26/5d-190)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +70億 &quot;&quot;(昨12/5d12)&quot;"/>
@@ -35,6 +35,7 @@
     <numFmt numFmtId="174" formatCode="0.0&quot;%&quot;"/>
     <numFmt numFmtId="175" formatCode="0&quot;%&quot;"/>
     <numFmt numFmtId="176" formatCode="#,##0.00;-#,##0.00"/>
+    <numFmt numFmtId="177" formatCode="0&quot; 檔 +69億 &quot;&quot;(昨12/5d12)&quot;"/>
   </numFmts>
   <fonts count="45">
     <font>
@@ -541,7 +542,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="222">
+  <cellXfs count="223">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1054,6 +1055,9 @@
     <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="177" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1139,12 +1143,12 @@
     <comment ref="D16" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 73.5%
-  • 領頭金額 125,231 萬
-  • 合計淨買 170,333 萬
+領頭大戶「陳族元」獨佔比 73.1%
+  • 領頭金額 122,814 萬
+  • 合計淨買 167,916 萬
   • 大戶數 11 位 (名義共識)
 判讀: 名義 11 位大戶共識,
-實質 1 人下注佔 74%,
+實質 1 人下注佔 73%,
 剩餘 10 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1152,9 +1156,9 @@
     <comment ref="D18" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 85.3%
-  • 領頭金額 113,167 萬
-  • 合計淨買 132,691 萬
+領頭大戶「陳族元」獨佔比 85.1%
+  • 領頭金額 111,125 萬
+  • 合計淨買 130,648 萬
   • 大戶數 11 位 (名義共識)
 判讀: 名義 11 位大戶共識,
 實質 1 人下注佔 85%,
@@ -1513,7 +1517,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 📌 一般共識 2327 / 4958 / 3189 (Q5 中性, 中性信號)  |  避開 — 除權息 27 檔: 1101, 1101B, 1470 ... | 明日恐處置 1 檔: 2303  |  訊號: 中性但 hot 多 (24 個信號 — 留意)</t>
+          <t>💡 📌 一般共識 2327 / 4958 / 3189 (Q5 中性, 中性信號)  |  避開 — 除權息 27 檔: 1101, 1101B, 1470 ... | 明日恐處置 5 檔: 3189/6213/8021...  |  訊號: 中性但 hot 多 (24 個信號 — 留意)</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1669,7 @@
         <v>11</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
@@ -1673,7 +1677,7 @@
         </is>
       </c>
       <c r="H16" s="18" t="n">
-        <v>125231</v>
+        <v>122814</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1695,7 +1699,7 @@
         <v>8</v>
       </c>
       <c r="N16" s="18" t="n">
-        <v>170333</v>
+        <v>167916</v>
       </c>
     </row>
     <row r="17">
@@ -1732,7 +1736,7 @@
         </is>
       </c>
       <c r="J17" s="19" t="n">
-        <v>27838</v>
+        <v>27775</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1746,7 +1750,7 @@
         <v>8</v>
       </c>
       <c r="N17" s="18" t="n">
-        <v>140869</v>
+        <v>140806</v>
       </c>
     </row>
     <row r="18">
@@ -1767,7 +1771,7 @@
         <v>11</v>
       </c>
       <c r="F18" s="16" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G18" s="17" t="inlineStr">
         <is>
@@ -1775,7 +1779,7 @@
         </is>
       </c>
       <c r="H18" s="18" t="n">
-        <v>113168</v>
+        <v>111125</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1797,7 +1801,7 @@
         <v>8</v>
       </c>
       <c r="N18" s="18" t="n">
-        <v>132691</v>
+        <v>130649</v>
       </c>
     </row>
     <row r="19">
@@ -1826,7 +1830,7 @@
         </is>
       </c>
       <c r="H19" s="18" t="n">
-        <v>14365</v>
+        <v>14362</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1848,7 +1852,7 @@
         <v>10</v>
       </c>
       <c r="N19" s="18" t="n">
-        <v>53132</v>
+        <v>53128</v>
       </c>
     </row>
     <row r="20">
@@ -1877,7 +1881,7 @@
         </is>
       </c>
       <c r="H20" s="18" t="n">
-        <v>10887</v>
+        <v>9953</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1899,7 +1903,7 @@
         <v>10</v>
       </c>
       <c r="N20" s="18" t="n">
-        <v>49708</v>
+        <v>48774</v>
       </c>
     </row>
     <row r="21">
@@ -1908,49 +1912,49 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2408</t>
+          <t>2409</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>📌 南亞科</t>
+          <t>📌 友達</t>
         </is>
       </c>
       <c r="E21" s="15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F21" s="16" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G21" s="17" t="inlineStr">
         <is>
+          <t>張濬安</t>
+        </is>
+      </c>
+      <c r="H21" s="18" t="n">
+        <v>9401</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
           <t>陳族元</t>
         </is>
       </c>
-      <c r="H21" s="18" t="n">
-        <v>10443</v>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>林滄海</t>
-        </is>
-      </c>
       <c r="J21" s="19" t="n">
-        <v>8128</v>
+        <v>7221</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>布哥</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="L21" s="19" t="n">
-        <v>5062</v>
+        <v>3786</v>
       </c>
       <c r="M21" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N21" s="18" t="n">
-        <v>39670</v>
+        <v>31236</v>
       </c>
     </row>
     <row r="22">
@@ -1959,49 +1963,49 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2409</t>
+          <t>2408</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>📌 友達</t>
+          <t>📌 南亞科</t>
         </is>
       </c>
       <c r="E22" s="15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F22" s="16" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="G22" s="17" t="inlineStr">
         <is>
-          <t>張濬安</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="H22" s="18" t="n">
-        <v>9401</v>
+        <v>8128</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>布哥</t>
         </is>
       </c>
       <c r="J22" s="19" t="n">
-        <v>7158</v>
+        <v>5062</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>竹科主力分點</t>
+          <t>強森</t>
         </is>
       </c>
       <c r="L22" s="19" t="n">
-        <v>3786</v>
+        <v>3597</v>
       </c>
       <c r="M22" s="20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N22" s="18" t="n">
-        <v>31173</v>
+        <v>30627</v>
       </c>
     </row>
     <row r="23">
@@ -2046,13 +2050,13 @@
         </is>
       </c>
       <c r="L23" s="19" t="n">
-        <v>2461</v>
+        <v>2478</v>
       </c>
       <c r="M23" s="20" t="n">
         <v>9</v>
       </c>
       <c r="N23" s="18" t="n">
-        <v>22879</v>
+        <v>22896</v>
       </c>
     </row>
     <row r="24">
@@ -2061,19 +2065,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>8299</t>
+          <t>6770</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>📌 群聯</t>
+          <t>📌 力積電</t>
         </is>
       </c>
       <c r="E24" s="15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F24" s="16" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G24" s="17" t="inlineStr">
         <is>
@@ -2081,29 +2085,29 @@
         </is>
       </c>
       <c r="H24" s="18" t="n">
-        <v>3930</v>
+        <v>4403</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>竹科主力分點</t>
+          <t>強森</t>
         </is>
       </c>
       <c r="J24" s="19" t="n">
-        <v>2952</v>
+        <v>2523</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>布哥</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="L24" s="19" t="n">
-        <v>2889</v>
+        <v>2250</v>
       </c>
       <c r="M24" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N24" s="18" t="n">
-        <v>17237</v>
+        <v>17231</v>
       </c>
     </row>
     <row r="25">
@@ -2112,27 +2116,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>6770</t>
+          <t>2357</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>📌 力積電</t>
+          <t>📌 華碩</t>
         </is>
       </c>
       <c r="E25" s="15" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
-          <t>張濬安</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="H25" s="18" t="n">
-        <v>4403</v>
+        <v>6021</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -2140,7 +2144,7 @@
         </is>
       </c>
       <c r="J25" s="19" t="n">
-        <v>2523</v>
+        <v>2551</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -2148,13 +2152,13 @@
         </is>
       </c>
       <c r="L25" s="19" t="n">
-        <v>2250</v>
+        <v>2204</v>
       </c>
       <c r="M25" s="20" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="N25" s="18" t="n">
-        <v>17167</v>
+        <v>17026</v>
       </c>
     </row>
     <row r="26">
@@ -2163,49 +2167,49 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2357</t>
+          <t>8299</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>📌 華碩</t>
+          <t>📌 群聯</t>
         </is>
       </c>
       <c r="E26" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F26" s="16" t="n">
         <v>15</v>
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
+          <t>張濬安</t>
+        </is>
+      </c>
+      <c r="H26" s="18" t="n">
+        <v>3930</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
           <t>竹科主力分點</t>
         </is>
       </c>
-      <c r="H26" s="18" t="n">
-        <v>6021</v>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>強森</t>
-        </is>
-      </c>
       <c r="J26" s="19" t="n">
-        <v>2551</v>
+        <v>2952</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>林滄海</t>
+          <t>布哥</t>
         </is>
       </c>
       <c r="L26" s="19" t="n">
-        <v>2204</v>
+        <v>2889</v>
       </c>
       <c r="M26" s="20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N26" s="18" t="n">
-        <v>16403</v>
+        <v>16578</v>
       </c>
     </row>
     <row r="27">
@@ -2234,7 +2238,7 @@
         </is>
       </c>
       <c r="H27" s="18" t="n">
-        <v>1310</v>
+        <v>1334</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2256,7 +2260,7 @@
         <v>10</v>
       </c>
       <c r="N27" s="18" t="n">
-        <v>5513</v>
+        <v>5538</v>
       </c>
     </row>
     <row r="28">
@@ -2274,10 +2278,10 @@
         </is>
       </c>
       <c r="E28" s="15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F28" s="16" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
@@ -2304,10 +2308,10 @@
         <v>302</v>
       </c>
       <c r="M28" s="20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N28" s="18" t="n">
-        <v>3124</v>
+        <v>3056</v>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
@@ -2332,7 +2336,7 @@
         </is>
       </c>
       <c r="G31" s="196" t="n">
-        <v>-67.94410000000001</v>
+        <v>-70.77464999999999</v>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1">
@@ -2341,7 +2345,7 @@
           <t>Q3 強共識股</t>
         </is>
       </c>
-      <c r="C32" s="197" t="n">
+      <c r="C32" s="222" t="n">
         <v>13</v>
       </c>
       <c r="F32" s="22" t="inlineStr">
@@ -2350,7 +2354,7 @@
         </is>
       </c>
       <c r="G32" s="198" t="n">
-        <v>0.206919138606294</v>
+        <v>0.2062267155802317</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
@@ -2429,11 +2433,11 @@
         </is>
       </c>
       <c r="D38" s="33" t="n">
-        <v>2850916</v>
+        <v>2826495</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>39.1%</t>
+          <t>38.9%</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2465,7 +2469,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>25.3%</t>
+          <t>25.4%</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2497,7 +2501,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -2621,7 +2625,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>民哥</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2631,12 +2635,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 12 檔新標的 (過去從沒買過)</t>
+          <t>民哥 今日買進 10 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>12 檔</t>
+          <t>10 檔</t>
         </is>
       </c>
     </row>
@@ -2648,7 +2652,7 @@
       </c>
       <c r="C48" s="41" t="inlineStr">
         <is>
-          <t>民哥</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D48" s="41" t="inlineStr">
@@ -2658,7 +2662,7 @@
       </c>
       <c r="E48" s="41" t="inlineStr">
         <is>
-          <t>民哥 今日買進 10 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 10 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F48" s="41" t="inlineStr">
@@ -2943,11 +2947,11 @@
         <v>40</v>
       </c>
       <c r="E61" t="n">
-        <v>4199746</v>
+        <v>4194968</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>陳族元 連續 40 天加碼 2327 (累計 4,199,746 萬)</t>
+          <t>陳族元 連續 40 天加碼 2327 (累計 4,194,968 萬)</t>
         </is>
       </c>
     </row>
@@ -3012,11 +3016,11 @@
         <v>24</v>
       </c>
       <c r="E64" s="41" t="n">
-        <v>2459724</v>
+        <v>2454739</v>
       </c>
       <c r="F64" s="41" t="inlineStr">
         <is>
-          <t>陳族元 連續 24 天加碼 2454 (累計 2,459,724 萬)</t>
+          <t>陳族元 連續 24 天加碼 2454 (累計 2,454,739 萬)</t>
         </is>
       </c>
     </row>
@@ -3058,11 +3062,11 @@
         <v>22</v>
       </c>
       <c r="E66" s="41" t="n">
-        <v>1077017</v>
+        <v>1071058</v>
       </c>
       <c r="F66" s="41" t="inlineStr">
         <is>
-          <t>陳族元 連續 22 天加碼 2408 (累計 1,077,017 萬)</t>
+          <t>陳族元 連續 22 天加碼 2408 (累計 1,071,058 萬)</t>
         </is>
       </c>
     </row>
@@ -3173,7 +3177,7 @@
         </is>
       </c>
       <c r="C72" s="33" t="n">
-        <v>2794292</v>
+        <v>2769537</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3200,7 +3204,7 @@
         <v>198077</v>
       </c>
       <c r="J72" s="202" t="n">
-        <v>0.285803447077483</v>
+        <v>0.2883579763176334</v>
       </c>
     </row>
     <row r="73">
@@ -5080,7 +5084,7 @@
     <row r="26">
       <c r="C26" s="69" t="inlineStr">
         <is>
-          <t>明日恐處置 1 檔 (2303)</t>
+          <t>明日恐處置 5 檔 (3189 / 6213 / 8021 ...)</t>
         </is>
       </c>
     </row>
@@ -5094,7 +5098,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="C29" s="70" t="inlineStr">
         <is>
-          <t>-68 億 淨買</t>
+          <t>-71 億 淨買</t>
         </is>
       </c>
     </row>
@@ -13653,29 +13657,29 @@
       </c>
       <c r="D189" s="128" t="inlineStr">
         <is>
-          <t>南亞科(2408)</t>
+          <t>聯電(2303)</t>
         </is>
       </c>
       <c r="E189" s="129" t="n">
-        <v>268</v>
+        <v>504</v>
       </c>
       <c r="F189" s="129" t="n">
-        <v>38</v>
+        <v>152</v>
       </c>
       <c r="G189" s="129" t="n">
-        <v>11302</v>
+        <v>8511</v>
       </c>
       <c r="H189" s="129" t="n">
-        <v>1610</v>
+        <v>2574</v>
       </c>
       <c r="I189" s="129" t="n">
-        <v>9692</v>
+        <v>5937</v>
       </c>
       <c r="J189" s="130" t="n">
-        <v>421.71</v>
+        <v>168.87</v>
       </c>
       <c r="K189" s="130" t="n">
-        <v>423.61</v>
+        <v>169.34</v>
       </c>
       <c r="L189" s="220">
         <f>F189*(K189-J189)</f>
@@ -13688,29 +13692,29 @@
       <c r="C190" s="131" t="n"/>
       <c r="D190" s="128" t="inlineStr">
         <is>
-          <t>聯電(2303)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="E190" s="129" t="n">
-        <v>498</v>
+        <v>260</v>
       </c>
       <c r="F190" s="129" t="n">
-        <v>152</v>
+        <v>37</v>
       </c>
       <c r="G190" s="129" t="n">
-        <v>8416</v>
+        <v>5343</v>
       </c>
       <c r="H190" s="129" t="n">
-        <v>2569</v>
+        <v>4694</v>
       </c>
       <c r="I190" s="129" t="n">
-        <v>5847</v>
+        <v>649</v>
       </c>
       <c r="J190" s="130" t="n">
-        <v>169</v>
+        <v>205.51</v>
       </c>
       <c r="K190" s="130" t="n">
-        <v>169</v>
+        <v>1268.51</v>
       </c>
       <c r="L190" s="220">
         <f>F190*(K190-J190)</f>
@@ -13723,31 +13727,31 @@
       <c r="C191" s="131" t="n"/>
       <c r="D191" s="128" t="inlineStr">
         <is>
-          <t>智邦(2345)</t>
+          <t>創見(2451)</t>
         </is>
       </c>
       <c r="E191" s="129" t="n">
-        <v>20</v>
+        <v>146</v>
       </c>
       <c r="F191" s="129" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G191" s="129" t="n">
-        <v>5230</v>
+        <v>3657</v>
       </c>
       <c r="H191" s="129" t="n">
-        <v>3343</v>
+        <v>200</v>
       </c>
       <c r="I191" s="129" t="n">
-        <v>1887</v>
+        <v>3457</v>
       </c>
       <c r="J191" s="130" t="n">
-        <v>2615.15</v>
+        <v>250.5</v>
       </c>
       <c r="K191" s="130" t="n">
-        <v>2571.38</v>
-      </c>
-      <c r="L191" s="219">
+        <v>250.5</v>
+      </c>
+      <c r="L191" s="220">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -13758,31 +13762,31 @@
       <c r="C192" s="131" t="n"/>
       <c r="D192" s="128" t="inlineStr">
         <is>
-          <t>聯發科(2454)</t>
+          <t>大立光(3008)</t>
         </is>
       </c>
       <c r="E192" s="129" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F192" s="129" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G192" s="129" t="n">
-        <v>4985</v>
+        <v>3561</v>
       </c>
       <c r="H192" s="129" t="n">
-        <v>4384</v>
+        <v>1864</v>
       </c>
       <c r="I192" s="129" t="n">
-        <v>601</v>
+        <v>1697</v>
       </c>
       <c r="J192" s="130" t="n">
-        <v>4531.73</v>
+        <v>4451.25</v>
       </c>
       <c r="K192" s="130" t="n">
-        <v>4384.4</v>
-      </c>
-      <c r="L192" s="219">
+        <v>4659</v>
+      </c>
+      <c r="L192" s="220">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -13793,29 +13797,29 @@
       <c r="C193" s="131" t="n"/>
       <c r="D193" s="128" t="inlineStr">
         <is>
-          <t>國巨*(2327)</t>
+          <t>欣興(3037)</t>
         </is>
       </c>
       <c r="E193" s="129" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="F193" s="129" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G193" s="129" t="n">
-        <v>4778</v>
+        <v>3462</v>
       </c>
       <c r="H193" s="129" t="n">
-        <v>2361</v>
+        <v>1447</v>
       </c>
       <c r="I193" s="129" t="n">
-        <v>2417</v>
+        <v>2015</v>
       </c>
       <c r="J193" s="130" t="n">
-        <v>1137.57</v>
+        <v>1049.24</v>
       </c>
       <c r="K193" s="130" t="n">
-        <v>1124.14</v>
+        <v>1033.79</v>
       </c>
       <c r="L193" s="219">
         <f>F193*(K193-J193)</f>
@@ -13828,31 +13832,31 @@
       <c r="C194" s="131" t="n"/>
       <c r="D194" s="128" t="inlineStr">
         <is>
-          <t>景碩(3189)</t>
+          <t>臻鼎-KY(4958)</t>
         </is>
       </c>
       <c r="E194" s="129" t="n">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="F194" s="129" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="G194" s="129" t="n">
-        <v>4152</v>
+        <v>3419</v>
       </c>
       <c r="H194" s="129" t="n">
-        <v>2110</v>
+        <v>1775</v>
       </c>
       <c r="I194" s="129" t="n">
-        <v>2042</v>
+        <v>1644</v>
       </c>
       <c r="J194" s="130" t="n">
-        <v>883.49</v>
+        <v>599.89</v>
       </c>
       <c r="K194" s="130" t="n">
-        <v>879.12</v>
-      </c>
-      <c r="L194" s="219">
+        <v>612.03</v>
+      </c>
+      <c r="L194" s="220">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -13867,27 +13871,27 @@
         </is>
       </c>
       <c r="E195" s="129" t="n">
-        <v>486</v>
+        <v>538</v>
       </c>
       <c r="F195" s="129" t="n">
-        <v>259</v>
+        <v>461</v>
       </c>
       <c r="G195" s="129" t="n">
-        <v>3761</v>
+        <v>3398</v>
       </c>
       <c r="H195" s="129" t="n">
-        <v>3227</v>
+        <v>1797</v>
       </c>
       <c r="I195" s="129" t="n">
-        <v>534</v>
+        <v>1601</v>
       </c>
       <c r="J195" s="130" t="n">
-        <v>77.38</v>
+        <v>63.15</v>
       </c>
       <c r="K195" s="130" t="n">
-        <v>124.59</v>
-      </c>
-      <c r="L195" s="220">
+        <v>38.97</v>
+      </c>
+      <c r="L195" s="219">
         <f>F195*(K195-J195)</f>
         <v/>
       </c>
@@ -13898,29 +13902,29 @@
       <c r="C196" s="131" t="n"/>
       <c r="D196" s="128" t="inlineStr">
         <is>
-          <t>創見(2451)</t>
+          <t>力積電(6770)</t>
         </is>
       </c>
       <c r="E196" s="129" t="n">
-        <v>148</v>
+        <v>364</v>
       </c>
       <c r="F196" s="129" t="n">
-        <v>8</v>
+        <v>234</v>
       </c>
       <c r="G196" s="129" t="n">
-        <v>3703</v>
+        <v>2702</v>
       </c>
       <c r="H196" s="129" t="n">
-        <v>205</v>
+        <v>1739</v>
       </c>
       <c r="I196" s="129" t="n">
-        <v>3498</v>
+        <v>963</v>
       </c>
       <c r="J196" s="130" t="n">
-        <v>250.2</v>
+        <v>74.22</v>
       </c>
       <c r="K196" s="130" t="n">
-        <v>256.5</v>
+        <v>74.31</v>
       </c>
       <c r="L196" s="220">
         <f>F196*(K196-J196)</f>
@@ -13933,31 +13937,31 @@
       <c r="C197" s="131" t="n"/>
       <c r="D197" s="128" t="inlineStr">
         <is>
-          <t>臻鼎-KY(4958)</t>
+          <t>華邦電(2344)</t>
         </is>
       </c>
       <c r="E197" s="129" t="n">
-        <v>55</v>
+        <v>149</v>
       </c>
       <c r="F197" s="129" t="n">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="G197" s="129" t="n">
-        <v>3188</v>
+        <v>2687</v>
       </c>
       <c r="H197" s="129" t="n">
-        <v>1481</v>
+        <v>1967</v>
       </c>
       <c r="I197" s="129" t="n">
-        <v>1707</v>
+        <v>720</v>
       </c>
       <c r="J197" s="130" t="n">
-        <v>579.64</v>
+        <v>180.36</v>
       </c>
       <c r="K197" s="130" t="n">
-        <v>510.59</v>
-      </c>
-      <c r="L197" s="219">
+        <v>312.25</v>
+      </c>
+      <c r="L197" s="220">
         <f>F197*(K197-J197)</f>
         <v/>
       </c>
@@ -13968,29 +13972,29 @@
       <c r="C198" s="131" t="n"/>
       <c r="D198" s="128" t="inlineStr">
         <is>
-          <t>華邦電(2344)</t>
+          <t>南電(8046)</t>
         </is>
       </c>
       <c r="E198" s="129" t="n">
-        <v>138</v>
+        <v>20</v>
       </c>
       <c r="F198" s="129" t="n">
-        <v>102</v>
+        <v>16</v>
       </c>
       <c r="G198" s="129" t="n">
-        <v>2888</v>
+        <v>2373</v>
       </c>
       <c r="H198" s="129" t="n">
-        <v>1234</v>
+        <v>1858</v>
       </c>
       <c r="I198" s="129" t="n">
-        <v>1654</v>
+        <v>515</v>
       </c>
       <c r="J198" s="130" t="n">
-        <v>209.28</v>
+        <v>1186.6</v>
       </c>
       <c r="K198" s="130" t="n">
-        <v>121.01</v>
+        <v>1161.19</v>
       </c>
       <c r="L198" s="219">
         <f>F198*(K198-J198)</f>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-07-02 01:13
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -1143,12 +1143,12 @@
     <comment ref="D16" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 73.1%
-  • 領頭金額 122,814 萬
-  • 合計淨買 167,916 萬
+領頭大戶「陳族元」獨佔比 73.5%
+  • 領頭金額 125,231 萬
+  • 合計淨買 170,333 萬
   • 大戶數 11 位 (名義共識)
 判讀: 名義 11 位大戶共識,
-實質 1 人下注佔 73%,
+實質 1 人下注佔 74%,
 剩餘 10 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1156,9 +1156,9 @@
     <comment ref="D18" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 85.1%
-  • 領頭金額 111,125 萬
-  • 合計淨買 130,648 萬
+領頭大戶「陳族元」獨佔比 85.3%
+  • 領頭金額 113,167 萬
+  • 合計淨買 132,691 萬
   • 大戶數 11 位 (名義共識)
 判讀: 名義 11 位大戶共識,
 實質 1 人下注佔 85%,
@@ -1669,7 +1669,7 @@
         <v>11</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
@@ -1677,7 +1677,7 @@
         </is>
       </c>
       <c r="H16" s="18" t="n">
-        <v>122814</v>
+        <v>125231</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1699,7 +1699,7 @@
         <v>8</v>
       </c>
       <c r="N16" s="18" t="n">
-        <v>167916</v>
+        <v>170333</v>
       </c>
     </row>
     <row r="17">
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="J17" s="19" t="n">
-        <v>27775</v>
+        <v>27838</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1750,7 +1750,7 @@
         <v>8</v>
       </c>
       <c r="N17" s="18" t="n">
-        <v>140806</v>
+        <v>140869</v>
       </c>
     </row>
     <row r="18">
@@ -1771,7 +1771,7 @@
         <v>11</v>
       </c>
       <c r="F18" s="16" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G18" s="17" t="inlineStr">
         <is>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="H18" s="18" t="n">
-        <v>111125</v>
+        <v>113168</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1801,7 +1801,7 @@
         <v>8</v>
       </c>
       <c r="N18" s="18" t="n">
-        <v>130649</v>
+        <v>132691</v>
       </c>
     </row>
     <row r="19">
@@ -1822,7 +1822,7 @@
         <v>13</v>
       </c>
       <c r="F19" s="16" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G19" s="17" t="inlineStr">
         <is>
@@ -1830,7 +1830,7 @@
         </is>
       </c>
       <c r="H19" s="18" t="n">
-        <v>14362</v>
+        <v>13571</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1852,7 +1852,7 @@
         <v>10</v>
       </c>
       <c r="N19" s="18" t="n">
-        <v>53128</v>
+        <v>52338</v>
       </c>
     </row>
     <row r="20">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="H20" s="18" t="n">
-        <v>9953</v>
+        <v>10887</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1903,7 +1903,7 @@
         <v>10</v>
       </c>
       <c r="N20" s="18" t="n">
-        <v>48774</v>
+        <v>49708</v>
       </c>
     </row>
     <row r="21">
@@ -1912,49 +1912,49 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2409</t>
+          <t>2408</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>📌 友達</t>
+          <t>📌 南亞科</t>
         </is>
       </c>
       <c r="E21" s="15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F21" s="16" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="G21" s="17" t="inlineStr">
         <is>
-          <t>張濬安</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="H21" s="18" t="n">
-        <v>9401</v>
+        <v>10443</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="J21" s="19" t="n">
-        <v>7221</v>
+        <v>8128</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>竹科主力分點</t>
+          <t>布哥</t>
         </is>
       </c>
       <c r="L21" s="19" t="n">
-        <v>3786</v>
+        <v>5062</v>
       </c>
       <c r="M21" s="20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N21" s="18" t="n">
-        <v>31236</v>
+        <v>39670</v>
       </c>
     </row>
     <row r="22">
@@ -1963,49 +1963,49 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2408</t>
+          <t>2409</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>📌 南亞科</t>
+          <t>📌 友達</t>
         </is>
       </c>
       <c r="E22" s="15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F22" s="16" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G22" s="17" t="inlineStr">
         <is>
-          <t>林滄海</t>
+          <t>張濬安</t>
         </is>
       </c>
       <c r="H22" s="18" t="n">
-        <v>8128</v>
+        <v>9401</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>布哥</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="J22" s="19" t="n">
-        <v>5062</v>
+        <v>6490</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>強森</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="L22" s="19" t="n">
-        <v>3597</v>
+        <v>3786</v>
       </c>
       <c r="M22" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N22" s="18" t="n">
-        <v>30627</v>
+        <v>30505</v>
       </c>
     </row>
     <row r="23">
@@ -2026,7 +2026,7 @@
         <v>12</v>
       </c>
       <c r="F23" s="16" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G23" s="17" t="inlineStr">
         <is>
@@ -2046,17 +2046,17 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>張濬安</t>
         </is>
       </c>
       <c r="L23" s="19" t="n">
-        <v>2478</v>
+        <v>1726</v>
       </c>
       <c r="M23" s="20" t="n">
         <v>9</v>
       </c>
       <c r="N23" s="18" t="n">
-        <v>22896</v>
+        <v>21324</v>
       </c>
     </row>
     <row r="24">
@@ -2065,19 +2065,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>6770</t>
+          <t>8299</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>📌 力積電</t>
+          <t>📌 群聯</t>
         </is>
       </c>
       <c r="E24" s="15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F24" s="16" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="G24" s="17" t="inlineStr">
         <is>
@@ -2085,29 +2085,29 @@
         </is>
       </c>
       <c r="H24" s="18" t="n">
-        <v>4403</v>
+        <v>3930</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>強森</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="J24" s="19" t="n">
-        <v>2523</v>
+        <v>2952</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>林滄海</t>
+          <t>布哥</t>
         </is>
       </c>
       <c r="L24" s="19" t="n">
-        <v>2250</v>
+        <v>2889</v>
       </c>
       <c r="M24" s="20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N24" s="18" t="n">
-        <v>17231</v>
+        <v>17237</v>
       </c>
     </row>
     <row r="25">
@@ -2128,7 +2128,7 @@
         <v>10</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
@@ -2158,7 +2158,7 @@
         <v>7</v>
       </c>
       <c r="N25" s="18" t="n">
-        <v>17026</v>
+        <v>16403</v>
       </c>
     </row>
     <row r="26">
@@ -2167,19 +2167,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>8299</t>
+          <t>6770</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>📌 群聯</t>
+          <t>📌 力積電</t>
         </is>
       </c>
       <c r="E26" s="15" t="n">
         <v>11</v>
       </c>
       <c r="F26" s="16" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
@@ -2187,29 +2187,29 @@
         </is>
       </c>
       <c r="H26" s="18" t="n">
-        <v>3930</v>
+        <v>4403</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>竹科主力分點</t>
+          <t>強森</t>
         </is>
       </c>
       <c r="J26" s="19" t="n">
-        <v>2952</v>
+        <v>2523</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>布哥</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="L26" s="19" t="n">
-        <v>2889</v>
+        <v>2250</v>
       </c>
       <c r="M26" s="20" t="n">
         <v>8</v>
       </c>
       <c r="N26" s="18" t="n">
-        <v>16578</v>
+        <v>16268</v>
       </c>
     </row>
     <row r="27">
@@ -2234,19 +2234,19 @@
       </c>
       <c r="G27" s="17" t="inlineStr">
         <is>
+          <t>強森</t>
+        </is>
+      </c>
+      <c r="H27" s="18" t="n">
+        <v>1004</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
           <t>陳族元</t>
         </is>
       </c>
-      <c r="H27" s="18" t="n">
-        <v>1334</v>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>強森</t>
-        </is>
-      </c>
       <c r="J27" s="19" t="n">
-        <v>1004</v>
+        <v>858</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -2260,7 +2260,7 @@
         <v>10</v>
       </c>
       <c r="N27" s="18" t="n">
-        <v>5538</v>
+        <v>5062</v>
       </c>
     </row>
     <row r="28">
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="G31" s="196" t="n">
-        <v>-70.77464999999999</v>
+        <v>-69.29268999999999</v>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1">
@@ -2345,7 +2345,7 @@
           <t>Q3 強共識股</t>
         </is>
       </c>
-      <c r="C32" s="222" t="n">
+      <c r="C32" s="197" t="n">
         <v>13</v>
       </c>
       <c r="F32" s="22" t="inlineStr">
@@ -2354,7 +2354,7 @@
         </is>
       </c>
       <c r="G32" s="198" t="n">
-        <v>0.2062267155802317</v>
+        <v>0.2064924530775332</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="D38" s="33" t="n">
-        <v>2826495</v>
+        <v>2833870</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>民哥</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2635,12 +2635,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>民哥 今日買進 10 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 11 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>10 檔</t>
+          <t>11 檔</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="C48" s="41" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>民哥</t>
         </is>
       </c>
       <c r="D48" s="41" t="inlineStr">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="E48" s="41" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 10 檔新標的 (過去從沒買過)</t>
+          <t>民哥 今日買進 10 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F48" s="41" t="inlineStr">
@@ -2947,11 +2947,11 @@
         <v>40</v>
       </c>
       <c r="E61" t="n">
-        <v>4194968</v>
+        <v>4199746</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>陳族元 連續 40 天加碼 2327 (累計 4,194,968 萬)</t>
+          <t>陳族元 連續 40 天加碼 2327 (累計 4,199,746 萬)</t>
         </is>
       </c>
     </row>
@@ -3016,11 +3016,11 @@
         <v>24</v>
       </c>
       <c r="E64" s="41" t="n">
-        <v>2454739</v>
+        <v>2459724</v>
       </c>
       <c r="F64" s="41" t="inlineStr">
         <is>
-          <t>陳族元 連續 24 天加碼 2454 (累計 2,454,739 萬)</t>
+          <t>陳族元 連續 24 天加碼 2454 (累計 2,459,724 萬)</t>
         </is>
       </c>
     </row>
@@ -3062,11 +3062,11 @@
         <v>22</v>
       </c>
       <c r="E66" s="41" t="n">
-        <v>1071058</v>
+        <v>1077017</v>
       </c>
       <c r="F66" s="41" t="inlineStr">
         <is>
-          <t>陳族元 連續 22 天加碼 2408 (累計 1,071,058 萬)</t>
+          <t>陳族元 連續 22 天加碼 2408 (累計 1,077,017 萬)</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3177,7 @@
         </is>
       </c>
       <c r="C72" s="33" t="n">
-        <v>2769537</v>
+        <v>2776908</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3204,7 +3204,7 @@
         <v>198077</v>
       </c>
       <c r="J72" s="202" t="n">
-        <v>0.2883579763176334</v>
+        <v>0.2875925512129766</v>
       </c>
     </row>
     <row r="73">
@@ -5098,7 +5098,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="C29" s="70" t="inlineStr">
         <is>
-          <t>-71 億 淨買</t>
+          <t>-69 億 淨買</t>
         </is>
       </c>
     </row>
@@ -13657,29 +13657,29 @@
       </c>
       <c r="D189" s="128" t="inlineStr">
         <is>
-          <t>聯電(2303)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="E189" s="129" t="n">
-        <v>504</v>
+        <v>260</v>
       </c>
       <c r="F189" s="129" t="n">
-        <v>152</v>
+        <v>37</v>
       </c>
       <c r="G189" s="129" t="n">
-        <v>8511</v>
+        <v>11302</v>
       </c>
       <c r="H189" s="129" t="n">
-        <v>2574</v>
+        <v>1610</v>
       </c>
       <c r="I189" s="129" t="n">
-        <v>5937</v>
+        <v>9692</v>
       </c>
       <c r="J189" s="130" t="n">
-        <v>168.87</v>
+        <v>434.69</v>
       </c>
       <c r="K189" s="130" t="n">
-        <v>169.34</v>
+        <v>435.05</v>
       </c>
       <c r="L189" s="220">
         <f>F189*(K189-J189)</f>
@@ -13692,31 +13692,31 @@
       <c r="C190" s="131" t="n"/>
       <c r="D190" s="128" t="inlineStr">
         <is>
-          <t>南亞科(2408)</t>
+          <t>智邦(2345)</t>
         </is>
       </c>
       <c r="E190" s="129" t="n">
-        <v>260</v>
+        <v>20</v>
       </c>
       <c r="F190" s="129" t="n">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="G190" s="129" t="n">
-        <v>5343</v>
+        <v>5230</v>
       </c>
       <c r="H190" s="129" t="n">
-        <v>4694</v>
+        <v>3343</v>
       </c>
       <c r="I190" s="129" t="n">
-        <v>649</v>
+        <v>1887</v>
       </c>
       <c r="J190" s="130" t="n">
-        <v>205.51</v>
+        <v>2615.15</v>
       </c>
       <c r="K190" s="130" t="n">
-        <v>1268.51</v>
-      </c>
-      <c r="L190" s="220">
+        <v>2571.38</v>
+      </c>
+      <c r="L190" s="219">
         <f>F190*(K190-J190)</f>
         <v/>
       </c>
@@ -13727,31 +13727,31 @@
       <c r="C191" s="131" t="n"/>
       <c r="D191" s="128" t="inlineStr">
         <is>
-          <t>創見(2451)</t>
+          <t>聯發科(2454)</t>
         </is>
       </c>
       <c r="E191" s="129" t="n">
-        <v>146</v>
+        <v>11</v>
       </c>
       <c r="F191" s="129" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G191" s="129" t="n">
-        <v>3657</v>
+        <v>4985</v>
       </c>
       <c r="H191" s="129" t="n">
-        <v>200</v>
+        <v>4384</v>
       </c>
       <c r="I191" s="129" t="n">
-        <v>3457</v>
+        <v>601</v>
       </c>
       <c r="J191" s="130" t="n">
-        <v>250.5</v>
+        <v>4531.73</v>
       </c>
       <c r="K191" s="130" t="n">
-        <v>250.5</v>
-      </c>
-      <c r="L191" s="220">
+        <v>4384.4</v>
+      </c>
+      <c r="L191" s="219">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -13762,31 +13762,31 @@
       <c r="C192" s="131" t="n"/>
       <c r="D192" s="128" t="inlineStr">
         <is>
-          <t>大立光(3008)</t>
+          <t>國巨*(2327)</t>
         </is>
       </c>
       <c r="E192" s="129" t="n">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="F192" s="129" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="G192" s="129" t="n">
-        <v>3561</v>
+        <v>4778</v>
       </c>
       <c r="H192" s="129" t="n">
-        <v>1864</v>
+        <v>2361</v>
       </c>
       <c r="I192" s="129" t="n">
-        <v>1697</v>
+        <v>2417</v>
       </c>
       <c r="J192" s="130" t="n">
-        <v>4451.25</v>
+        <v>1137.57</v>
       </c>
       <c r="K192" s="130" t="n">
-        <v>4659</v>
-      </c>
-      <c r="L192" s="220">
+        <v>1124.14</v>
+      </c>
+      <c r="L192" s="219">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -13797,29 +13797,29 @@
       <c r="C193" s="131" t="n"/>
       <c r="D193" s="128" t="inlineStr">
         <is>
-          <t>欣興(3037)</t>
+          <t>景碩(3189)</t>
         </is>
       </c>
       <c r="E193" s="129" t="n">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="F193" s="129" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G193" s="129" t="n">
-        <v>3462</v>
+        <v>4152</v>
       </c>
       <c r="H193" s="129" t="n">
-        <v>1447</v>
+        <v>2110</v>
       </c>
       <c r="I193" s="129" t="n">
-        <v>2015</v>
+        <v>2042</v>
       </c>
       <c r="J193" s="130" t="n">
-        <v>1049.24</v>
+        <v>883.49</v>
       </c>
       <c r="K193" s="130" t="n">
-        <v>1033.79</v>
+        <v>879.12</v>
       </c>
       <c r="L193" s="219">
         <f>F193*(K193-J193)</f>
@@ -13832,29 +13832,29 @@
       <c r="C194" s="131" t="n"/>
       <c r="D194" s="128" t="inlineStr">
         <is>
-          <t>臻鼎-KY(4958)</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E194" s="129" t="n">
-        <v>57</v>
+        <v>538</v>
       </c>
       <c r="F194" s="129" t="n">
-        <v>29</v>
+        <v>461</v>
       </c>
       <c r="G194" s="129" t="n">
-        <v>3419</v>
+        <v>3761</v>
       </c>
       <c r="H194" s="129" t="n">
-        <v>1775</v>
+        <v>3227</v>
       </c>
       <c r="I194" s="129" t="n">
-        <v>1644</v>
+        <v>534</v>
       </c>
       <c r="J194" s="130" t="n">
-        <v>599.89</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="K194" s="130" t="n">
-        <v>612.03</v>
+        <v>70</v>
       </c>
       <c r="L194" s="220">
         <f>F194*(K194-J194)</f>
@@ -13867,31 +13867,31 @@
       <c r="C195" s="131" t="n"/>
       <c r="D195" s="128" t="inlineStr">
         <is>
-          <t>群創(3481)</t>
+          <t>創見(2451)</t>
         </is>
       </c>
       <c r="E195" s="129" t="n">
-        <v>538</v>
+        <v>146</v>
       </c>
       <c r="F195" s="129" t="n">
-        <v>461</v>
+        <v>8</v>
       </c>
       <c r="G195" s="129" t="n">
-        <v>3398</v>
+        <v>3703</v>
       </c>
       <c r="H195" s="129" t="n">
-        <v>1797</v>
+        <v>205</v>
       </c>
       <c r="I195" s="129" t="n">
-        <v>1601</v>
+        <v>3498</v>
       </c>
       <c r="J195" s="130" t="n">
-        <v>63.15</v>
+        <v>253.63</v>
       </c>
       <c r="K195" s="130" t="n">
-        <v>38.97</v>
-      </c>
-      <c r="L195" s="219">
+        <v>256.5</v>
+      </c>
+      <c r="L195" s="220">
         <f>F195*(K195-J195)</f>
         <v/>
       </c>
@@ -13902,31 +13902,31 @@
       <c r="C196" s="131" t="n"/>
       <c r="D196" s="128" t="inlineStr">
         <is>
-          <t>力積電(6770)</t>
+          <t>臻鼎-KY(4958)</t>
         </is>
       </c>
       <c r="E196" s="129" t="n">
-        <v>364</v>
+        <v>53</v>
       </c>
       <c r="F196" s="129" t="n">
-        <v>234</v>
+        <v>25</v>
       </c>
       <c r="G196" s="129" t="n">
-        <v>2702</v>
+        <v>3188</v>
       </c>
       <c r="H196" s="129" t="n">
-        <v>1739</v>
+        <v>1481</v>
       </c>
       <c r="I196" s="129" t="n">
-        <v>963</v>
+        <v>1707</v>
       </c>
       <c r="J196" s="130" t="n">
-        <v>74.22</v>
+        <v>601.51</v>
       </c>
       <c r="K196" s="130" t="n">
-        <v>74.31</v>
-      </c>
-      <c r="L196" s="220">
+        <v>592.28</v>
+      </c>
+      <c r="L196" s="219">
         <f>F196*(K196-J196)</f>
         <v/>
       </c>
@@ -13937,29 +13937,29 @@
       <c r="C197" s="131" t="n"/>
       <c r="D197" s="128" t="inlineStr">
         <is>
-          <t>華邦電(2344)</t>
+          <t>友達(2409)</t>
         </is>
       </c>
       <c r="E197" s="129" t="n">
-        <v>149</v>
+        <v>963</v>
       </c>
       <c r="F197" s="129" t="n">
-        <v>63</v>
+        <v>910</v>
       </c>
       <c r="G197" s="129" t="n">
-        <v>2687</v>
+        <v>2952</v>
       </c>
       <c r="H197" s="129" t="n">
-        <v>1967</v>
+        <v>2789</v>
       </c>
       <c r="I197" s="129" t="n">
-        <v>720</v>
+        <v>163</v>
       </c>
       <c r="J197" s="130" t="n">
-        <v>180.36</v>
+        <v>30.65</v>
       </c>
       <c r="K197" s="130" t="n">
-        <v>312.25</v>
+        <v>30.65</v>
       </c>
       <c r="L197" s="220">
         <f>F197*(K197-J197)</f>
@@ -13972,31 +13972,31 @@
       <c r="C198" s="131" t="n"/>
       <c r="D198" s="128" t="inlineStr">
         <is>
-          <t>南電(8046)</t>
+          <t>華邦電(2344)</t>
         </is>
       </c>
       <c r="E198" s="129" t="n">
-        <v>20</v>
+        <v>149</v>
       </c>
       <c r="F198" s="129" t="n">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="G198" s="129" t="n">
-        <v>2373</v>
+        <v>2888</v>
       </c>
       <c r="H198" s="129" t="n">
-        <v>1858</v>
+        <v>1234</v>
       </c>
       <c r="I198" s="129" t="n">
-        <v>515</v>
+        <v>1654</v>
       </c>
       <c r="J198" s="130" t="n">
-        <v>1186.6</v>
+        <v>193.83</v>
       </c>
       <c r="K198" s="130" t="n">
-        <v>1161.19</v>
-      </c>
-      <c r="L198" s="219">
+        <v>195.92</v>
+      </c>
+      <c r="L198" s="220">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-07-02 01:47
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -1822,7 +1822,7 @@
         <v>13</v>
       </c>
       <c r="F19" s="16" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G19" s="17" t="inlineStr">
         <is>
@@ -1830,7 +1830,7 @@
         </is>
       </c>
       <c r="H19" s="18" t="n">
-        <v>13571</v>
+        <v>14365</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1852,7 +1852,7 @@
         <v>10</v>
       </c>
       <c r="N19" s="18" t="n">
-        <v>52338</v>
+        <v>53132</v>
       </c>
     </row>
     <row r="20">
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="J22" s="19" t="n">
-        <v>6490</v>
+        <v>7158</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -2005,7 +2005,7 @@
         <v>9</v>
       </c>
       <c r="N22" s="18" t="n">
-        <v>30505</v>
+        <v>31173</v>
       </c>
     </row>
     <row r="23">
@@ -2026,7 +2026,7 @@
         <v>12</v>
       </c>
       <c r="F23" s="16" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G23" s="17" t="inlineStr">
         <is>
@@ -2046,17 +2046,17 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>張濬安</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="L23" s="19" t="n">
-        <v>1726</v>
+        <v>2461</v>
       </c>
       <c r="M23" s="20" t="n">
         <v>9</v>
       </c>
       <c r="N23" s="18" t="n">
-        <v>21324</v>
+        <v>22879</v>
       </c>
     </row>
     <row r="24">
@@ -2116,27 +2116,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2357</t>
+          <t>6770</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>📌 華碩</t>
+          <t>📌 力積電</t>
         </is>
       </c>
       <c r="E25" s="15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
-          <t>竹科主力分點</t>
+          <t>張濬安</t>
         </is>
       </c>
       <c r="H25" s="18" t="n">
-        <v>6021</v>
+        <v>4403</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -2144,7 +2144,7 @@
         </is>
       </c>
       <c r="J25" s="19" t="n">
-        <v>2551</v>
+        <v>2523</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -2152,13 +2152,13 @@
         </is>
       </c>
       <c r="L25" s="19" t="n">
-        <v>2204</v>
+        <v>2250</v>
       </c>
       <c r="M25" s="20" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N25" s="18" t="n">
-        <v>16403</v>
+        <v>17167</v>
       </c>
     </row>
     <row r="26">
@@ -2167,27 +2167,27 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>6770</t>
+          <t>2357</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>📌 力積電</t>
+          <t>📌 華碩</t>
         </is>
       </c>
       <c r="E26" s="15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F26" s="16" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
-          <t>張濬安</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="H26" s="18" t="n">
-        <v>4403</v>
+        <v>6021</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -2195,7 +2195,7 @@
         </is>
       </c>
       <c r="J26" s="19" t="n">
-        <v>2523</v>
+        <v>2551</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -2203,13 +2203,13 @@
         </is>
       </c>
       <c r="L26" s="19" t="n">
-        <v>2250</v>
+        <v>2204</v>
       </c>
       <c r="M26" s="20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N26" s="18" t="n">
-        <v>16268</v>
+        <v>16403</v>
       </c>
     </row>
     <row r="27">
@@ -2234,19 +2234,19 @@
       </c>
       <c r="G27" s="17" t="inlineStr">
         <is>
+          <t>陳族元</t>
+        </is>
+      </c>
+      <c r="H27" s="18" t="n">
+        <v>1310</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
           <t>強森</t>
         </is>
       </c>
-      <c r="H27" s="18" t="n">
+      <c r="J27" s="19" t="n">
         <v>1004</v>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>陳族元</t>
-        </is>
-      </c>
-      <c r="J27" s="19" t="n">
-        <v>858</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -2260,7 +2260,7 @@
         <v>10</v>
       </c>
       <c r="N27" s="18" t="n">
-        <v>5062</v>
+        <v>5513</v>
       </c>
     </row>
     <row r="28">
@@ -2278,10 +2278,10 @@
         </is>
       </c>
       <c r="E28" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F28" s="16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
@@ -2308,10 +2308,10 @@
         <v>302</v>
       </c>
       <c r="M28" s="20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N28" s="18" t="n">
-        <v>3056</v>
+        <v>3124</v>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="G31" s="196" t="n">
-        <v>-69.29268999999999</v>
+        <v>-67.94410000000001</v>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1">
@@ -2354,7 +2354,7 @@
         </is>
       </c>
       <c r="G32" s="198" t="n">
-        <v>0.2064924530775332</v>
+        <v>0.2069969164823522</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
@@ -2433,11 +2433,11 @@
         </is>
       </c>
       <c r="D38" s="33" t="n">
-        <v>2833870</v>
+        <v>2850916</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>38.9%</t>
+          <t>39.1%</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>25.4%</t>
+          <t>25.3%</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2635,12 +2635,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 11 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 12 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>11 檔</t>
+          <t>12 檔</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3177,7 @@
         </is>
       </c>
       <c r="C72" s="33" t="n">
-        <v>2776908</v>
+        <v>2794292</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3204,7 +3204,7 @@
         <v>198077</v>
       </c>
       <c r="J72" s="202" t="n">
-        <v>0.2875925512129766</v>
+        <v>0.285803447077483</v>
       </c>
     </row>
     <row r="73">
@@ -5098,7 +5098,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="C29" s="70" t="inlineStr">
         <is>
-          <t>-69 億 淨買</t>
+          <t>-68 億 淨買</t>
         </is>
       </c>
     </row>
@@ -13661,10 +13661,10 @@
         </is>
       </c>
       <c r="E189" s="129" t="n">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="F189" s="129" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G189" s="129" t="n">
         <v>11302</v>
@@ -13676,10 +13676,10 @@
         <v>9692</v>
       </c>
       <c r="J189" s="130" t="n">
-        <v>434.69</v>
+        <v>421.71</v>
       </c>
       <c r="K189" s="130" t="n">
-        <v>435.05</v>
+        <v>423.61</v>
       </c>
       <c r="L189" s="220">
         <f>F189*(K189-J189)</f>
@@ -13692,31 +13692,31 @@
       <c r="C190" s="131" t="n"/>
       <c r="D190" s="128" t="inlineStr">
         <is>
-          <t>智邦(2345)</t>
+          <t>聯電(2303)</t>
         </is>
       </c>
       <c r="E190" s="129" t="n">
-        <v>20</v>
+        <v>498</v>
       </c>
       <c r="F190" s="129" t="n">
-        <v>13</v>
+        <v>152</v>
       </c>
       <c r="G190" s="129" t="n">
-        <v>5230</v>
+        <v>8416</v>
       </c>
       <c r="H190" s="129" t="n">
-        <v>3343</v>
+        <v>2569</v>
       </c>
       <c r="I190" s="129" t="n">
-        <v>1887</v>
+        <v>5847</v>
       </c>
       <c r="J190" s="130" t="n">
-        <v>2615.15</v>
+        <v>169</v>
       </c>
       <c r="K190" s="130" t="n">
-        <v>2571.38</v>
-      </c>
-      <c r="L190" s="219">
+        <v>169</v>
+      </c>
+      <c r="L190" s="220">
         <f>F190*(K190-J190)</f>
         <v/>
       </c>
@@ -13727,29 +13727,29 @@
       <c r="C191" s="131" t="n"/>
       <c r="D191" s="128" t="inlineStr">
         <is>
-          <t>聯發科(2454)</t>
+          <t>智邦(2345)</t>
         </is>
       </c>
       <c r="E191" s="129" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F191" s="129" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G191" s="129" t="n">
-        <v>4985</v>
+        <v>5230</v>
       </c>
       <c r="H191" s="129" t="n">
-        <v>4384</v>
+        <v>3343</v>
       </c>
       <c r="I191" s="129" t="n">
-        <v>601</v>
+        <v>1887</v>
       </c>
       <c r="J191" s="130" t="n">
-        <v>4531.73</v>
+        <v>2615.15</v>
       </c>
       <c r="K191" s="130" t="n">
-        <v>4384.4</v>
+        <v>2571.38</v>
       </c>
       <c r="L191" s="219">
         <f>F191*(K191-J191)</f>
@@ -13762,29 +13762,29 @@
       <c r="C192" s="131" t="n"/>
       <c r="D192" s="128" t="inlineStr">
         <is>
-          <t>國巨*(2327)</t>
+          <t>聯發科(2454)</t>
         </is>
       </c>
       <c r="E192" s="129" t="n">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="F192" s="129" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="G192" s="129" t="n">
-        <v>4778</v>
+        <v>4985</v>
       </c>
       <c r="H192" s="129" t="n">
-        <v>2361</v>
+        <v>4384</v>
       </c>
       <c r="I192" s="129" t="n">
-        <v>2417</v>
+        <v>601</v>
       </c>
       <c r="J192" s="130" t="n">
-        <v>1137.57</v>
+        <v>4531.73</v>
       </c>
       <c r="K192" s="130" t="n">
-        <v>1124.14</v>
+        <v>4384.4</v>
       </c>
       <c r="L192" s="219">
         <f>F192*(K192-J192)</f>
@@ -13797,29 +13797,29 @@
       <c r="C193" s="131" t="n"/>
       <c r="D193" s="128" t="inlineStr">
         <is>
-          <t>景碩(3189)</t>
+          <t>國巨*(2327)</t>
         </is>
       </c>
       <c r="E193" s="129" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="F193" s="129" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G193" s="129" t="n">
-        <v>4152</v>
+        <v>4778</v>
       </c>
       <c r="H193" s="129" t="n">
-        <v>2110</v>
+        <v>2361</v>
       </c>
       <c r="I193" s="129" t="n">
-        <v>2042</v>
+        <v>2417</v>
       </c>
       <c r="J193" s="130" t="n">
-        <v>883.49</v>
+        <v>1137.57</v>
       </c>
       <c r="K193" s="130" t="n">
-        <v>879.12</v>
+        <v>1124.14</v>
       </c>
       <c r="L193" s="219">
         <f>F193*(K193-J193)</f>
@@ -13832,31 +13832,31 @@
       <c r="C194" s="131" t="n"/>
       <c r="D194" s="128" t="inlineStr">
         <is>
-          <t>群創(3481)</t>
+          <t>景碩(3189)</t>
         </is>
       </c>
       <c r="E194" s="129" t="n">
-        <v>538</v>
+        <v>47</v>
       </c>
       <c r="F194" s="129" t="n">
-        <v>461</v>
+        <v>24</v>
       </c>
       <c r="G194" s="129" t="n">
-        <v>3761</v>
+        <v>4152</v>
       </c>
       <c r="H194" s="129" t="n">
-        <v>3227</v>
+        <v>2110</v>
       </c>
       <c r="I194" s="129" t="n">
-        <v>534</v>
+        <v>2042</v>
       </c>
       <c r="J194" s="130" t="n">
-        <v>69.90000000000001</v>
+        <v>883.49</v>
       </c>
       <c r="K194" s="130" t="n">
-        <v>70</v>
-      </c>
-      <c r="L194" s="220">
+        <v>879.12</v>
+      </c>
+      <c r="L194" s="219">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -13867,29 +13867,29 @@
       <c r="C195" s="131" t="n"/>
       <c r="D195" s="128" t="inlineStr">
         <is>
-          <t>創見(2451)</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E195" s="129" t="n">
-        <v>146</v>
+        <v>486</v>
       </c>
       <c r="F195" s="129" t="n">
-        <v>8</v>
+        <v>259</v>
       </c>
       <c r="G195" s="129" t="n">
-        <v>3703</v>
+        <v>3761</v>
       </c>
       <c r="H195" s="129" t="n">
-        <v>205</v>
+        <v>3227</v>
       </c>
       <c r="I195" s="129" t="n">
-        <v>3498</v>
+        <v>534</v>
       </c>
       <c r="J195" s="130" t="n">
-        <v>253.63</v>
+        <v>77.38</v>
       </c>
       <c r="K195" s="130" t="n">
-        <v>256.5</v>
+        <v>124.59</v>
       </c>
       <c r="L195" s="220">
         <f>F195*(K195-J195)</f>
@@ -13902,31 +13902,31 @@
       <c r="C196" s="131" t="n"/>
       <c r="D196" s="128" t="inlineStr">
         <is>
-          <t>臻鼎-KY(4958)</t>
+          <t>創見(2451)</t>
         </is>
       </c>
       <c r="E196" s="129" t="n">
-        <v>53</v>
+        <v>148</v>
       </c>
       <c r="F196" s="129" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="G196" s="129" t="n">
-        <v>3188</v>
+        <v>3703</v>
       </c>
       <c r="H196" s="129" t="n">
-        <v>1481</v>
+        <v>205</v>
       </c>
       <c r="I196" s="129" t="n">
-        <v>1707</v>
+        <v>3498</v>
       </c>
       <c r="J196" s="130" t="n">
-        <v>601.51</v>
+        <v>250.2</v>
       </c>
       <c r="K196" s="130" t="n">
-        <v>592.28</v>
-      </c>
-      <c r="L196" s="219">
+        <v>256.5</v>
+      </c>
+      <c r="L196" s="220">
         <f>F196*(K196-J196)</f>
         <v/>
       </c>
@@ -13937,31 +13937,31 @@
       <c r="C197" s="131" t="n"/>
       <c r="D197" s="128" t="inlineStr">
         <is>
-          <t>友達(2409)</t>
+          <t>臻鼎-KY(4958)</t>
         </is>
       </c>
       <c r="E197" s="129" t="n">
-        <v>963</v>
+        <v>55</v>
       </c>
       <c r="F197" s="129" t="n">
-        <v>910</v>
+        <v>29</v>
       </c>
       <c r="G197" s="129" t="n">
-        <v>2952</v>
+        <v>3188</v>
       </c>
       <c r="H197" s="129" t="n">
-        <v>2789</v>
+        <v>1481</v>
       </c>
       <c r="I197" s="129" t="n">
-        <v>163</v>
+        <v>1707</v>
       </c>
       <c r="J197" s="130" t="n">
-        <v>30.65</v>
+        <v>579.64</v>
       </c>
       <c r="K197" s="130" t="n">
-        <v>30.65</v>
-      </c>
-      <c r="L197" s="220">
+        <v>510.59</v>
+      </c>
+      <c r="L197" s="219">
         <f>F197*(K197-J197)</f>
         <v/>
       </c>
@@ -13976,10 +13976,10 @@
         </is>
       </c>
       <c r="E198" s="129" t="n">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="F198" s="129" t="n">
-        <v>63</v>
+        <v>102</v>
       </c>
       <c r="G198" s="129" t="n">
         <v>2888</v>
@@ -13991,12 +13991,12 @@
         <v>1654</v>
       </c>
       <c r="J198" s="130" t="n">
-        <v>193.83</v>
+        <v>209.28</v>
       </c>
       <c r="K198" s="130" t="n">
-        <v>195.92</v>
-      </c>
-      <c r="L198" s="220">
+        <v>121.01</v>
+      </c>
+      <c r="L198" s="219">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-07-03 00:40
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="18">
+  <numFmts count="19">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨+26/5d-190)&quot;;-0&quot; 億 (昨+26/5d-190)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +70億 &quot;&quot;(昨12/5d12)&quot;"/>
@@ -41,8 +41,9 @@
     <numFmt numFmtId="179" formatCode="0&quot; 檔 +105億 &quot;&quot;(昨13/5d12)&quot;"/>
     <numFmt numFmtId="180" formatCode="0.0%&quot; 市-1418億 &quot;&quot;(昨21/5d18)&quot;"/>
     <numFmt numFmtId="181" formatCode="&quot;📅 明日預測 ↑ 偏多 &quot;0.0&quot;% 信心 — P/C Ratio 主推 — 3 檔焦點&quot;"/>
+    <numFmt numFmtId="182" formatCode="0.0%&quot; 市-1416億 &quot;&quot;(昨21/5d18)&quot;"/>
   </numFmts>
-  <fonts count="51">
+  <fonts count="52">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -334,6 +335,12 @@
       <color rgb="FFB45309"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Noto Sans TC"/>
+      <i val="1"/>
+      <color rgb="FF10B981"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="48">
     <fill>
@@ -588,7 +595,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="236">
+  <cellXfs count="238">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1133,6 +1140,10 @@
     <xf numFmtId="175" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="182" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1556,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N135"/>
+  <dimension ref="B2:N121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1592,7 +1603,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 📌 一般共識 2330 / 2454 / 5483 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 除權息 30 檔: 00939, 00984D, 1452 ... | 明日恐處置 5 檔: 3189/6213/8021...  |  訊號: 強偏多 (Q5 67.1%, hot=24)</t>
+          <t>💡 📌 一般共識 2330 / 2454 / 5483 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 明日恐處置 9 檔: 1447/1617/3055...  |  訊號: 強偏多 (Q5 67.1%, hot=24)</t>
         </is>
       </c>
     </row>
@@ -2275,8 +2286,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G29" s="225" t="n">
-        <v>0.2110509342257378</v>
+      <c r="G29" s="236" t="n">
+        <v>0.2106659514045904</v>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
@@ -3576,7 +3587,7 @@
     <row r="83" ht="22" customHeight="1">
       <c r="B83" s="59" t="inlineStr">
         <is>
-          <t>▍ G. 注意股 (資料日 20260701)</t>
+          <t>▍ G. 注意股 (資料日 20260703)</t>
         </is>
       </c>
     </row>
@@ -3608,755 +3619,769 @@
       </c>
     </row>
     <row r="85">
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>059570</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>強茂凱基5B購03</t>
-        </is>
-      </c>
-      <c r="D85" t="n">
-        <v>1</v>
-      </c>
-      <c r="E85" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>-----</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="B86" s="41" t="inlineStr">
-        <is>
-          <t>1435</t>
-        </is>
-      </c>
-      <c r="C86" s="41" t="inlineStr">
-        <is>
-          <t>中福</t>
-        </is>
-      </c>
-      <c r="D86" s="41" t="n">
-        <v>1</v>
-      </c>
-      <c r="E86" s="41" t="n">
-        <v>30.05</v>
-      </c>
-      <c r="F86" s="41" t="inlineStr">
-        <is>
-          <t>-----</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>1444</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>力麗</t>
-        </is>
-      </c>
-      <c r="D87" t="n">
-        <v>1</v>
-      </c>
-      <c r="E87" t="n">
-        <v>9.35</v>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>-----</t>
+      <c r="B85" s="237" t="inlineStr">
+        <is>
+          <t>✅ 今日無新增注意股 (市場無異常波動標的)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>▍ H. 借券賣出 Top 15 (機構級反向力量, 資料日 20260702)</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="B88" s="41" t="inlineStr">
-        <is>
-          <t>1447</t>
-        </is>
-      </c>
-      <c r="C88" s="41" t="inlineStr">
-        <is>
-          <t>力鵬</t>
-        </is>
-      </c>
-      <c r="D88" s="41" t="n">
-        <v>1</v>
-      </c>
-      <c r="E88" s="41" t="n">
-        <v>8.27</v>
-      </c>
-      <c r="F88" s="41" t="inlineStr">
-        <is>
-          <t>-----</t>
+      <c r="B88" s="12" t="inlineStr">
+        <is>
+          <t>代號</t>
+        </is>
+      </c>
+      <c r="C88" s="12" t="inlineStr">
+        <is>
+          <t>名稱</t>
+        </is>
+      </c>
+      <c r="D88" s="12" t="inlineStr">
+        <is>
+          <t>借券張數</t>
+        </is>
+      </c>
+      <c r="E88" s="12" t="inlineStr">
+        <is>
+          <t>融券張數</t>
+        </is>
+      </c>
+      <c r="F88" s="12" t="inlineStr">
+        <is>
+          <t>ratio</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="B89" t="inlineStr">
         <is>
-          <t>1617</t>
+          <t>6770</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>榮星</t>
-        </is>
-      </c>
-      <c r="D89" t="n">
+          <t>力積電</t>
+        </is>
+      </c>
+      <c r="D89" s="33" t="n">
+        <v>17785</v>
+      </c>
+      <c r="E89" s="33" t="n">
+        <v>1160</v>
+      </c>
+      <c r="F89" s="206" t="n">
+        <v>15.33</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="47" t="inlineStr">
+        <is>
+          <t>🔴 2886</t>
+        </is>
+      </c>
+      <c r="C90" s="41" t="inlineStr">
+        <is>
+          <t>兆豐金</t>
+        </is>
+      </c>
+      <c r="D90" s="62" t="n">
+        <v>14055</v>
+      </c>
+      <c r="E90" s="62" t="n">
         <v>1</v>
       </c>
-      <c r="E89" t="n">
-        <v>22.85</v>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>25.97</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="B90" s="41" t="inlineStr">
-        <is>
-          <t>1710</t>
-        </is>
-      </c>
-      <c r="C90" s="41" t="inlineStr">
-        <is>
-          <t>東聯</t>
-        </is>
-      </c>
-      <c r="D90" s="41" t="n">
-        <v>1</v>
-      </c>
-      <c r="E90" s="41" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="F90" s="41" t="inlineStr">
-        <is>
-          <t>-----</t>
-        </is>
+      <c r="F90" s="204" t="n">
+        <v>14055</v>
       </c>
     </row>
     <row r="91">
       <c r="B91" t="inlineStr">
         <is>
-          <t>1718</t>
+          <t>00981A</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>中纖</t>
-        </is>
-      </c>
-      <c r="D91" t="n">
+          <t>主動統一台股增長</t>
+        </is>
+      </c>
+      <c r="D91" s="33" t="n">
+        <v>11517</v>
+      </c>
+      <c r="E91" s="33" t="n">
+        <v>514</v>
+      </c>
+      <c r="F91" s="206" t="n">
+        <v>22.41</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="47" t="inlineStr">
+        <is>
+          <t>🔴 2891</t>
+        </is>
+      </c>
+      <c r="C92" s="41" t="inlineStr">
+        <is>
+          <t>中信金</t>
+        </is>
+      </c>
+      <c r="D92" s="62" t="n">
+        <v>8917</v>
+      </c>
+      <c r="E92" s="62" t="n">
         <v>1</v>
       </c>
-      <c r="E91" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>51.67</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="B92" s="41" t="inlineStr">
-        <is>
-          <t>2243</t>
-        </is>
-      </c>
-      <c r="C92" s="41" t="inlineStr">
-        <is>
-          <t>宏旭-KY</t>
-        </is>
-      </c>
-      <c r="D92" s="41" t="n">
-        <v>1</v>
-      </c>
-      <c r="E92" s="41" t="n">
-        <v>62</v>
-      </c>
-      <c r="F92" s="41" t="inlineStr">
-        <is>
-          <t>24.90</t>
-        </is>
+      <c r="F92" s="204" t="n">
+        <v>8917</v>
       </c>
     </row>
     <row r="93">
       <c r="B93" t="inlineStr">
         <is>
-          <t>2303</t>
+          <t>2317</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>聯電</t>
-        </is>
-      </c>
-      <c r="D93" t="n">
-        <v>1</v>
-      </c>
-      <c r="E93" t="n">
-        <v>169</v>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>42.46</t>
-        </is>
+          <t>鴻海</t>
+        </is>
+      </c>
+      <c r="D93" s="33" t="n">
+        <v>6897</v>
+      </c>
+      <c r="E93" s="33" t="n">
+        <v>24</v>
+      </c>
+      <c r="F93" s="206" t="n">
+        <v>287.38</v>
       </c>
     </row>
     <row r="94">
       <c r="B94" s="41" t="inlineStr">
         <is>
-          <t>2345</t>
+          <t>2313</t>
         </is>
       </c>
       <c r="C94" s="41" t="inlineStr">
         <is>
-          <t>智邦</t>
-        </is>
-      </c>
-      <c r="D94" s="41" t="n">
-        <v>1</v>
-      </c>
-      <c r="E94" s="41" t="n">
-        <v>2660</v>
-      </c>
-      <c r="F94" s="41" t="inlineStr">
-        <is>
-          <t>50.30</t>
-        </is>
+          <t>華通</t>
+        </is>
+      </c>
+      <c r="D94" s="62" t="n">
+        <v>6176</v>
+      </c>
+      <c r="E94" s="62" t="n">
+        <v>103</v>
+      </c>
+      <c r="F94" s="205" t="n">
+        <v>59.96</v>
       </c>
     </row>
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
-          <t>2363</t>
+          <t>4904</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>矽統</t>
-        </is>
-      </c>
-      <c r="D95" t="n">
-        <v>1</v>
-      </c>
-      <c r="E95" t="n">
-        <v>73.5</v>
+          <t>遠傳</t>
+        </is>
+      </c>
+      <c r="D95" s="33" t="n">
+        <v>5181</v>
+      </c>
+      <c r="E95" s="33" t="n">
+        <v>0</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>43.24</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="B96" s="41" t="inlineStr">
         <is>
-          <t>2375</t>
+          <t>2880</t>
         </is>
       </c>
       <c r="C96" s="41" t="inlineStr">
         <is>
-          <t>凱美</t>
-        </is>
-      </c>
-      <c r="D96" s="41" t="n">
-        <v>1</v>
-      </c>
-      <c r="E96" s="41" t="n">
-        <v>232.5</v>
+          <t>華南金</t>
+        </is>
+      </c>
+      <c r="D96" s="62" t="n">
+        <v>4899</v>
+      </c>
+      <c r="E96" s="62" t="n">
+        <v>0</v>
       </c>
       <c r="F96" s="41" t="inlineStr">
         <is>
-          <t>70.67</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="B97" t="inlineStr">
         <is>
-          <t>2406</t>
+          <t>3231</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>國碩</t>
-        </is>
-      </c>
-      <c r="D97" t="n">
+          <t>緯創</t>
+        </is>
+      </c>
+      <c r="D97" s="33" t="n">
+        <v>4880</v>
+      </c>
+      <c r="E97" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="B98" s="47" t="inlineStr">
+        <is>
+          <t>🔴 0056</t>
+        </is>
+      </c>
+      <c r="C98" s="41" t="inlineStr">
+        <is>
+          <t>元大高股息</t>
+        </is>
+      </c>
+      <c r="D98" s="62" t="n">
+        <v>4538</v>
+      </c>
+      <c r="E98" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="F98" s="204" t="n">
+        <v>1134.5</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" s="46" t="inlineStr">
+        <is>
+          <t>🔴 2892</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>第一金</t>
+        </is>
+      </c>
+      <c r="D99" s="33" t="n">
+        <v>4271</v>
+      </c>
+      <c r="E99" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="E97" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>-----</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="B98" s="41" t="inlineStr">
-        <is>
-          <t>2484</t>
-        </is>
-      </c>
-      <c r="C98" s="41" t="inlineStr">
-        <is>
-          <t>希華</t>
-        </is>
-      </c>
-      <c r="D98" s="41" t="n">
+      <c r="F99" s="203" t="n">
+        <v>4271</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" s="47" t="inlineStr">
+        <is>
+          <t>🔴 2412</t>
+        </is>
+      </c>
+      <c r="C100" s="41" t="inlineStr">
+        <is>
+          <t>中華電</t>
+        </is>
+      </c>
+      <c r="D100" s="62" t="n">
+        <v>4249</v>
+      </c>
+      <c r="E100" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="F100" s="204" t="n">
+        <v>2124.5</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" s="46" t="inlineStr">
+        <is>
+          <t>🔴 1101</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>台泥</t>
+        </is>
+      </c>
+      <c r="D101" s="33" t="n">
+        <v>4130</v>
+      </c>
+      <c r="E101" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="E98" s="41" t="n">
-        <v>79.8</v>
-      </c>
-      <c r="F98" s="41" t="inlineStr">
-        <is>
-          <t>107.84</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>3023</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>信邦</t>
-        </is>
-      </c>
-      <c r="D99" t="n">
-        <v>1</v>
-      </c>
-      <c r="E99" t="n">
-        <v>333</v>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>26.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="22" customHeight="1">
-      <c r="B101" s="4" t="inlineStr">
-        <is>
-          <t>▍ H. 借券賣出 Top 15 (機構級反向力量, 資料日 20260701)</t>
-        </is>
+      <c r="F101" s="203" t="n">
+        <v>4130</v>
       </c>
     </row>
     <row r="102">
-      <c r="B102" s="12" t="inlineStr">
+      <c r="B102" s="41" t="inlineStr">
+        <is>
+          <t>8112</t>
+        </is>
+      </c>
+      <c r="C102" s="41" t="inlineStr">
+        <is>
+          <t>至上</t>
+        </is>
+      </c>
+      <c r="D102" s="62" t="n">
+        <v>4099</v>
+      </c>
+      <c r="E102" s="62" t="n">
+        <v>0</v>
+      </c>
+      <c r="F102" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>8422</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>可寧衛*</t>
+        </is>
+      </c>
+      <c r="D103" s="33" t="n">
+        <v>3773</v>
+      </c>
+      <c r="E103" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="B105" s="65" t="inlineStr">
+        <is>
+          <t>▍ I. 未來 30 天除權息 (有效 258 檔, 已剔除過期)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" s="60" t="inlineStr">
+        <is>
+          <t>除權息日</t>
+        </is>
+      </c>
+      <c r="C106" s="60" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C102" s="12" t="inlineStr">
+      <c r="D106" s="60" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D102" s="12" t="inlineStr">
-        <is>
-          <t>借券張數</t>
-        </is>
-      </c>
-      <c r="E102" s="12" t="inlineStr">
-        <is>
-          <t>融券張數</t>
-        </is>
-      </c>
-      <c r="F102" s="12" t="inlineStr">
-        <is>
-          <t>ratio</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="B103" s="46" t="inlineStr">
-        <is>
-          <t>🔴 2887</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>台新新光金</t>
-        </is>
-      </c>
-      <c r="D103" s="33" t="n">
-        <v>13846</v>
-      </c>
-      <c r="E103" s="33" t="n">
-        <v>3</v>
-      </c>
-      <c r="F103" s="203" t="n">
-        <v>4615.33</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="B104" s="41" t="inlineStr">
-        <is>
-          <t>2891</t>
-        </is>
-      </c>
-      <c r="C104" s="41" t="inlineStr">
-        <is>
-          <t>中信金</t>
-        </is>
-      </c>
-      <c r="D104" s="62" t="n">
-        <v>12974</v>
-      </c>
-      <c r="E104" s="62" t="n">
-        <v>0</v>
-      </c>
-      <c r="F104" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>2890</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>永豐金</t>
-        </is>
-      </c>
-      <c r="D105" s="33" t="n">
-        <v>11153</v>
-      </c>
-      <c r="E105" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="B106" s="47" t="inlineStr">
-        <is>
-          <t>🔴 3231</t>
-        </is>
-      </c>
-      <c r="C106" s="41" t="inlineStr">
-        <is>
-          <t>緯創</t>
-        </is>
-      </c>
-      <c r="D106" s="62" t="n">
-        <v>11039</v>
-      </c>
-      <c r="E106" s="62" t="n">
-        <v>3</v>
-      </c>
-      <c r="F106" s="204" t="n">
-        <v>3679.67</v>
+      <c r="E106" s="60" t="inlineStr">
+        <is>
+          <t>類型</t>
+        </is>
+      </c>
+      <c r="F106" s="60" t="inlineStr">
+        <is>
+          <t>現金股利</t>
+        </is>
       </c>
     </row>
     <row r="107">
-      <c r="B107" s="46" t="inlineStr">
-        <is>
-          <t>🔴 2002</t>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>20260703</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>中鋼</t>
-        </is>
-      </c>
-      <c r="D107" s="33" t="n">
-        <v>8477</v>
-      </c>
-      <c r="E107" s="33" t="n">
-        <v>5</v>
-      </c>
-      <c r="F107" s="203" t="n">
-        <v>1695.4</v>
+          <t>1455</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>集盛</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>0.16</v>
       </c>
     </row>
     <row r="108">
       <c r="B108" s="41" t="inlineStr">
         <is>
-          <t>2344</t>
+          <t>20260703</t>
         </is>
       </c>
       <c r="C108" s="41" t="inlineStr">
         <is>
-          <t>華邦電</t>
-        </is>
-      </c>
-      <c r="D108" s="62" t="n">
-        <v>7892</v>
-      </c>
-      <c r="E108" s="62" t="n">
-        <v>451</v>
-      </c>
-      <c r="F108" s="205" t="n">
-        <v>17.5</v>
+          <t>1730</t>
+        </is>
+      </c>
+      <c r="D108" s="41" t="inlineStr">
+        <is>
+          <t>花仙子</t>
+        </is>
+      </c>
+      <c r="E108" s="41" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F108" s="41" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>1718</t>
+          <t>20260703</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>中纖</t>
-        </is>
-      </c>
-      <c r="D109" s="33" t="n">
-        <v>7786</v>
-      </c>
-      <c r="E109" s="33" t="n">
-        <v>437</v>
-      </c>
-      <c r="F109" s="206" t="n">
-        <v>17.82</v>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>中鋼構</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>2.4</v>
       </c>
     </row>
     <row r="110">
-      <c r="B110" s="47" t="inlineStr">
-        <is>
-          <t>🔴 1101</t>
+      <c r="B110" s="41" t="inlineStr">
+        <is>
+          <t>20260703</t>
         </is>
       </c>
       <c r="C110" s="41" t="inlineStr">
         <is>
-          <t>台泥</t>
-        </is>
-      </c>
-      <c r="D110" s="62" t="n">
-        <v>7348</v>
-      </c>
-      <c r="E110" s="62" t="n">
-        <v>2</v>
-      </c>
-      <c r="F110" s="204" t="n">
-        <v>3674</v>
+          <t>2425</t>
+        </is>
+      </c>
+      <c r="D110" s="41" t="inlineStr">
+        <is>
+          <t>承啟</t>
+        </is>
+      </c>
+      <c r="E110" s="41" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F110" s="41" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="111">
-      <c r="B111" s="46" t="inlineStr">
-        <is>
-          <t>🔴 0056</t>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>20260703</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>元大高股息</t>
-        </is>
-      </c>
-      <c r="D111" s="33" t="n">
-        <v>7238</v>
-      </c>
-      <c r="E111" s="33" t="n">
-        <v>4</v>
-      </c>
-      <c r="F111" s="203" t="n">
-        <v>1809.5</v>
+          <t>2838A</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>聯邦銀甲特</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>2.630625</v>
       </c>
     </row>
     <row r="112">
       <c r="B112" s="41" t="inlineStr">
         <is>
-          <t>2317</t>
+          <t>20260703</t>
         </is>
       </c>
       <c r="C112" s="41" t="inlineStr">
         <is>
-          <t>鴻海</t>
-        </is>
-      </c>
-      <c r="D112" s="62" t="n">
-        <v>6334</v>
-      </c>
-      <c r="E112" s="62" t="n">
-        <v>0</v>
-      </c>
-      <c r="F112" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2945</t>
+        </is>
+      </c>
+      <c r="D112" s="41" t="inlineStr">
+        <is>
+          <t>三商家購</t>
+        </is>
+      </c>
+      <c r="E112" s="41" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F112" s="41" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="113">
-      <c r="B113" s="46" t="inlineStr">
-        <is>
-          <t>🔴 2886</t>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>20260703</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>兆豐金</t>
-        </is>
-      </c>
-      <c r="D113" s="33" t="n">
-        <v>6035</v>
-      </c>
-      <c r="E113" s="33" t="n">
-        <v>5</v>
-      </c>
-      <c r="F113" s="203" t="n">
-        <v>1207</v>
+          <t>3711</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>日月光投控</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>6.584838</v>
       </c>
     </row>
     <row r="114">
       <c r="B114" s="41" t="inlineStr">
         <is>
-          <t>2312</t>
+          <t>20260703</t>
         </is>
       </c>
       <c r="C114" s="41" t="inlineStr">
         <is>
-          <t>金寶</t>
-        </is>
-      </c>
-      <c r="D114" s="62" t="n">
-        <v>5782</v>
-      </c>
-      <c r="E114" s="62" t="n">
-        <v>74</v>
-      </c>
-      <c r="F114" s="205" t="n">
-        <v>78.14</v>
+          <t>910861</t>
+        </is>
+      </c>
+      <c r="D114" s="41" t="inlineStr">
+        <is>
+          <t>神州-DR</t>
+        </is>
+      </c>
+      <c r="E114" s="41" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F114" s="41" t="n">
+        <v>0.072018</v>
       </c>
     </row>
     <row r="115">
       <c r="B115" t="inlineStr">
         <is>
-          <t>2892</t>
+          <t>20260706</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>第一金</t>
-        </is>
-      </c>
-      <c r="D115" s="33" t="n">
-        <v>5366</v>
-      </c>
-      <c r="E115" s="33" t="n">
-        <v>278</v>
-      </c>
-      <c r="F115" s="206" t="n">
-        <v>19.3</v>
+          <t>00946</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>群益科技高息成長</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>0.058</v>
       </c>
     </row>
     <row r="116">
       <c r="B116" s="41" t="inlineStr">
         <is>
-          <t>9904</t>
+          <t>20260706</t>
         </is>
       </c>
       <c r="C116" s="41" t="inlineStr">
         <is>
-          <t>寶成</t>
-        </is>
-      </c>
-      <c r="D116" s="62" t="n">
-        <v>5179</v>
-      </c>
-      <c r="E116" s="62" t="n">
-        <v>0</v>
-      </c>
-      <c r="F116" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>00953B</t>
+        </is>
+      </c>
+      <c r="D116" s="41" t="inlineStr">
+        <is>
+          <t>群益優選非投等債</t>
+        </is>
+      </c>
+      <c r="E116" s="41" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F116" s="41" t="n">
+        <v>0.061</v>
       </c>
     </row>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
-          <t>2489</t>
+          <t>20260706</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>瑞軒</t>
-        </is>
-      </c>
-      <c r="D117" s="33" t="n">
-        <v>5112</v>
-      </c>
-      <c r="E117" s="33" t="n">
-        <v>602</v>
-      </c>
-      <c r="F117" s="206" t="n">
-        <v>8.49</v>
-      </c>
-    </row>
-    <row r="119" ht="22" customHeight="1">
-      <c r="B119" s="65" t="inlineStr">
-        <is>
-          <t>▍ I. 未來 30 天除權息 (有效 279 檔, 已剔除過期)</t>
-        </is>
+          <t>00985B</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>群益ESG投等債0-5</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>0.048</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" s="41" t="inlineStr">
+        <is>
+          <t>20260706</t>
+        </is>
+      </c>
+      <c r="C118" s="41" t="inlineStr">
+        <is>
+          <t>00997A</t>
+        </is>
+      </c>
+      <c r="D118" s="41" t="inlineStr">
+        <is>
+          <t>主動群益美國增長</t>
+        </is>
+      </c>
+      <c r="E118" s="41" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F118" s="41" t="n">
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>20260706</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>1307</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>三芳</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>2.2</v>
       </c>
     </row>
     <row r="120">
-      <c r="B120" s="60" t="inlineStr">
-        <is>
-          <t>除權息日</t>
-        </is>
-      </c>
-      <c r="C120" s="60" t="inlineStr">
-        <is>
-          <t>代號</t>
-        </is>
-      </c>
-      <c r="D120" s="60" t="inlineStr">
-        <is>
-          <t>名稱</t>
-        </is>
-      </c>
-      <c r="E120" s="60" t="inlineStr">
-        <is>
-          <t>類型</t>
-        </is>
-      </c>
-      <c r="F120" s="60" t="inlineStr">
-        <is>
-          <t>現金股利</t>
-        </is>
+      <c r="B120" s="41" t="inlineStr">
+        <is>
+          <t>20260706</t>
+        </is>
+      </c>
+      <c r="C120" s="41" t="inlineStr">
+        <is>
+          <t>2373</t>
+        </is>
+      </c>
+      <c r="D120" s="41" t="inlineStr">
+        <is>
+          <t>震旦行</t>
+        </is>
+      </c>
+      <c r="E120" s="41" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F120" s="41" t="n">
+        <v>3.7</v>
       </c>
     </row>
     <row r="121">
       <c r="B121" t="inlineStr">
         <is>
-          <t>20260702</t>
+          <t>20260706</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>00939</t>
+          <t>2474</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>統一台灣高息動能</t>
+          <t>可成</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -4365,370 +4390,19 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>0.125</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="B122" s="41" t="inlineStr">
-        <is>
-          <t>20260702</t>
-        </is>
-      </c>
-      <c r="C122" s="41" t="inlineStr">
-        <is>
-          <t>00984D</t>
-        </is>
-      </c>
-      <c r="D122" s="41" t="inlineStr">
-        <is>
-          <t>主動聯博全球非投</t>
-        </is>
-      </c>
-      <c r="E122" s="41" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F122" s="41" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>20260702</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>1452</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>宏益</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F123" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="B124" s="41" t="inlineStr">
-        <is>
-          <t>20260702</t>
-        </is>
-      </c>
-      <c r="C124" s="41" t="inlineStr">
-        <is>
-          <t>1612</t>
-        </is>
-      </c>
-      <c r="D124" s="41" t="inlineStr">
-        <is>
-          <t>宏泰</t>
-        </is>
-      </c>
-      <c r="E124" s="41" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F124" s="41" t="n">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>20260702</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>1752</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>南光</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F125" t="n">
-        <v>1.6</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="B126" s="41" t="inlineStr">
-        <is>
-          <t>20260702</t>
-        </is>
-      </c>
-      <c r="C126" s="41" t="inlineStr">
-        <is>
-          <t>1789</t>
-        </is>
-      </c>
-      <c r="D126" s="41" t="inlineStr">
-        <is>
-          <t>神隆</t>
-        </is>
-      </c>
-      <c r="E126" s="41" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F126" s="41" t="n">
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>20260702</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>2010</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>春源</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F127" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="B128" s="41" t="inlineStr">
-        <is>
-          <t>20260702</t>
-        </is>
-      </c>
-      <c r="C128" s="41" t="inlineStr">
-        <is>
-          <t>2317</t>
-        </is>
-      </c>
-      <c r="D128" s="41" t="inlineStr">
-        <is>
-          <t>鴻海</t>
-        </is>
-      </c>
-      <c r="E128" s="41" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F128" s="41" t="n">
-        <v>7.171792</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>20260702</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>2354</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>鴻準</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F129" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="B130" s="41" t="inlineStr">
-        <is>
-          <t>20260702</t>
-        </is>
-      </c>
-      <c r="C130" s="41" t="inlineStr">
-        <is>
-          <t>2433</t>
-        </is>
-      </c>
-      <c r="D130" s="41" t="inlineStr">
-        <is>
-          <t>互盛電</t>
-        </is>
-      </c>
-      <c r="E130" s="41" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F130" s="41" t="n">
-        <v>2.7</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>20260702</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>2462</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>良得電</t>
-        </is>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F131" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="B132" s="41" t="inlineStr">
-        <is>
-          <t>20260702</t>
-        </is>
-      </c>
-      <c r="C132" s="41" t="inlineStr">
-        <is>
-          <t>2607</t>
-        </is>
-      </c>
-      <c r="D132" s="41" t="inlineStr">
-        <is>
-          <t>榮運</t>
-        </is>
-      </c>
-      <c r="E132" s="41" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F132" s="41" t="n">
-        <v>2.7</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>20260702</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>2753</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>八方雲集</t>
-        </is>
-      </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F133" t="n">
-        <v>7.5</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="B134" s="41" t="inlineStr">
-        <is>
-          <t>20260702</t>
-        </is>
-      </c>
-      <c r="C134" s="41" t="inlineStr">
-        <is>
-          <t>2820</t>
-        </is>
-      </c>
-      <c r="D134" s="41" t="inlineStr">
-        <is>
-          <t>華票</t>
-        </is>
-      </c>
-      <c r="E134" s="41" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F134" s="41" t="n">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>20260702</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>3006</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr">
-        <is>
-          <t>晶豪科</t>
-        </is>
-      </c>
-      <c r="E135" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F135" t="n">
-        <v>1</v>
+        <v>7.113868</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="29">
     <mergeCell ref="G28:I28"/>
     <mergeCell ref="B67:J67"/>
     <mergeCell ref="B9:N9"/>
     <mergeCell ref="B42:J42"/>
     <mergeCell ref="B54:F54"/>
-    <mergeCell ref="B101:J101"/>
     <mergeCell ref="B33:E33"/>
     <mergeCell ref="B30:N30"/>
-    <mergeCell ref="B119:J119"/>
+    <mergeCell ref="B87:J87"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="B4:N4"/>
     <mergeCell ref="B7:N7"/>
@@ -4747,6 +4421,8 @@
     <mergeCell ref="B27:J27"/>
     <mergeCell ref="C28:D28"/>
     <mergeCell ref="B56:J56"/>
+    <mergeCell ref="B85:F85"/>
+    <mergeCell ref="B105:J105"/>
     <mergeCell ref="B10:N10"/>
   </mergeCells>
   <conditionalFormatting sqref="N16:N25">
@@ -4821,17 +4497,8 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D85:D99">
+  <conditionalFormatting sqref="D89:D103">
     <cfRule type="dataBar" priority="9">
-      <dataBar minLength="5" maxLength="90" showValue="1">
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFB300"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D103:D117">
-    <cfRule type="dataBar" priority="10">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -4839,8 +4506,8 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F103:F117">
-    <cfRule type="dataBar" priority="11">
+  <conditionalFormatting sqref="F89:F103">
+    <cfRule type="dataBar" priority="10">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -5039,16 +4706,16 @@
       </c>
     </row>
     <row r="32">
-      <c r="C32" s="69" t="inlineStr">
-        <is>
-          <t>除權息 30 檔 (00939 / 00984D / 1452 ...)</t>
+      <c r="C32" s="71" t="inlineStr">
+        <is>
+          <t>今日無除權息</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="C33" s="69" t="inlineStr">
         <is>
-          <t>明日恐處置 5 檔 (3189 / 6213 / 8021 ...)</t>
+          <t>明日恐處置 9 檔 (1447 / 1617 / 3055 ...)</t>
         </is>
       </c>
     </row>
@@ -11095,7 +10762,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="B3" s="98" t="inlineStr">
         <is>
-          <t>大牌分析師 近 51/51 交易日出手 2465 次 (521 檔), 風格分布: 隔日沖近似 39% / 當沖 13% / 留倉 48%, 漲停命中 5% (其中 🔒鎖漲停 4%), 前 5 大集中 24%, 長線部位 61% (35 檔), ⚠️ 處置股部位 14% (48 檔), 📦 連續囤貨 29 檔 (最長 13 天 009816, 4 檔仍 active)。 主軸: 高頻交易/持續進場/📦 連續囤貨。</t>
+          <t>大牌分析師 近 51/51 交易日出手 2465 次 (521 檔), 風格分布: 隔日沖近似 39% / 當沖 13% / 留倉 48%, 漲停命中 5% (其中 🔒鎖漲停 4%), 前 5 大集中 24%, 長線部位 61% (35 檔), ⚠️ 處置股部位 11% (42 檔), 📦 連續囤貨 29 檔 (最長 13 天 009816, 4 檔仍 active)。 主軸: 高頻交易/持續進場/📦 連續囤貨。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-07-03 01:34
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="19">
+  <numFmts count="20">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨+26/5d-190)&quot;;-0&quot; 億 (昨+26/5d-190)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +70億 &quot;&quot;(昨12/5d12)&quot;"/>
@@ -42,6 +42,7 @@
     <numFmt numFmtId="180" formatCode="0.0%&quot; 市-1418億 &quot;&quot;(昨21/5d18)&quot;"/>
     <numFmt numFmtId="181" formatCode="&quot;📅 明日預測 ↑ 偏多 &quot;0.0&quot;% 信心 — P/C Ratio 主推 — 3 檔焦點&quot;"/>
     <numFmt numFmtId="182" formatCode="0.0%&quot; 市-1416億 &quot;&quot;(昨21/5d18)&quot;"/>
+    <numFmt numFmtId="183" formatCode="0.0%&quot; 市-1417億 &quot;&quot;(昨21/5d18)&quot;"/>
   </numFmts>
   <fonts count="52">
     <font>
@@ -595,7 +596,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="238">
+  <cellXfs count="239">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1144,6 +1145,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="51" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="183" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2238,13 +2242,13 @@
         </is>
       </c>
       <c r="L25" s="19" t="n">
-        <v>528</v>
+        <v>479</v>
       </c>
       <c r="M25" s="20" t="n">
         <v>7</v>
       </c>
       <c r="N25" s="18" t="n">
-        <v>6291</v>
+        <v>6242</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -2269,7 +2273,7 @@
         </is>
       </c>
       <c r="G28" s="223" t="n">
-        <v>16.67531</v>
+        <v>16.23846</v>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
@@ -2286,8 +2290,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G29" s="236" t="n">
-        <v>0.2106659514045904</v>
+      <c r="G29" s="238" t="n">
+        <v>0.2107734731758731</v>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
@@ -2398,11 +2402,11 @@
         </is>
       </c>
       <c r="D36" s="33" t="n">
-        <v>1199489</v>
+        <v>1202887</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>22.8%</t>
+          <t>22.9%</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2434,7 +2438,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -3147,7 +3151,7 @@
         </is>
       </c>
       <c r="C70" s="33" t="n">
-        <v>1108795</v>
+        <v>1111948</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3174,7 +3178,7 @@
         <v>73050</v>
       </c>
       <c r="J70" s="202" t="n">
-        <v>0.2383021249907783</v>
+        <v>0.2376265538388181</v>
       </c>
     </row>
     <row r="71">
@@ -4729,7 +4733,7 @@
     <row r="36" ht="22" customHeight="1">
       <c r="C36" s="226" t="inlineStr">
         <is>
-          <t>+17 億 淨買</t>
+          <t>+16 億 淨買</t>
         </is>
       </c>
     </row>
@@ -18532,10 +18536,10 @@
         </is>
       </c>
       <c r="E195" s="129" t="n">
-        <v>271</v>
+        <v>147</v>
       </c>
       <c r="F195" s="129" t="n">
-        <v>175</v>
+        <v>40</v>
       </c>
       <c r="G195" s="129" t="n">
         <v>2924</v>
@@ -18547,12 +18551,12 @@
         <v>1091</v>
       </c>
       <c r="J195" s="130" t="n">
-        <v>107.91</v>
+        <v>198.93</v>
       </c>
       <c r="K195" s="130" t="n">
-        <v>104.74</v>
-      </c>
-      <c r="L195" s="219">
+        <v>458.23</v>
+      </c>
+      <c r="L195" s="220">
         <f>F195*(K195-J195)</f>
         <v/>
       </c>
@@ -18567,10 +18571,10 @@
         </is>
       </c>
       <c r="E196" s="129" t="n">
-        <v>204</v>
+        <v>71</v>
       </c>
       <c r="F196" s="129" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G196" s="129" t="n">
         <v>2793</v>
@@ -18582,12 +18586,12 @@
         <v>2181</v>
       </c>
       <c r="J196" s="130" t="n">
-        <v>136.91</v>
+        <v>393.38</v>
       </c>
       <c r="K196" s="130" t="n">
-        <v>145.74</v>
-      </c>
-      <c r="L196" s="220">
+        <v>139.11</v>
+      </c>
+      <c r="L196" s="219">
         <f>F196*(K196-J196)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-07-03 08:46
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -1635,7 +1635,7 @@
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>🟡 跟單實際淨報酬 (扣 0.585% 成本): 淨 hit 116/228 = 51% | 平均 +0.92% | 中位 +0.08% | 累積 +211% — 勉強損益兩平</t>
+          <t>🟡 跟單實際淨報酬 (扣 0.585% 成本): 淨 hit 116/228 = 51% | 平均 +0.92% | 中位 +0.08% | 累積 +210% — 勉強損益兩平</t>
         </is>
       </c>
     </row>
@@ -2242,13 +2242,13 @@
         </is>
       </c>
       <c r="L25" s="19" t="n">
-        <v>479</v>
+        <v>528</v>
       </c>
       <c r="M25" s="20" t="n">
         <v>7</v>
       </c>
       <c r="N25" s="18" t="n">
-        <v>6242</v>
+        <v>6291</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -2273,7 +2273,7 @@
         </is>
       </c>
       <c r="G28" s="223" t="n">
-        <v>16.23846</v>
+        <v>16.67345</v>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
@@ -2290,8 +2290,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G29" s="238" t="n">
-        <v>0.2107734731758731</v>
+      <c r="G29" s="225" t="n">
+        <v>0.2110515210419748</v>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
@@ -2402,11 +2402,11 @@
         </is>
       </c>
       <c r="D36" s="33" t="n">
-        <v>1202887</v>
+        <v>1199489</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>22.9%</t>
+          <t>22.8%</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="C47" s="41" t="inlineStr">
         <is>
-          <t>林滄海</t>
+          <t>民哥</t>
         </is>
       </c>
       <c r="D47" s="41" t="inlineStr">
@@ -2653,12 +2653,12 @@
       </c>
       <c r="E47" s="41" t="inlineStr">
         <is>
-          <t>林滄海 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>民哥 今日買進 7 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F47" s="41" t="inlineStr">
         <is>
-          <t>6 檔</t>
+          <t>7 檔</t>
         </is>
       </c>
     </row>
@@ -2670,7 +2670,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>民哥</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>民哥 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>林滄海 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -3151,7 +3151,7 @@
         </is>
       </c>
       <c r="C70" s="33" t="n">
-        <v>1111948</v>
+        <v>1108795</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3178,7 +3178,7 @@
         <v>73050</v>
       </c>
       <c r="J70" s="202" t="n">
-        <v>0.2376265538388181</v>
+        <v>0.2383021249907783</v>
       </c>
     </row>
     <row r="71">
@@ -3373,7 +3373,7 @@
         </is>
       </c>
       <c r="C76" s="33" t="n">
-        <v>132255</v>
+        <v>132292</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         <v>9264</v>
       </c>
       <c r="J76" s="202" t="n">
-        <v>0.3169780476942631</v>
+        <v>0.3168893938328802</v>
       </c>
     </row>
     <row r="77">
@@ -4733,7 +4733,7 @@
     <row r="36" ht="22" customHeight="1">
       <c r="C36" s="226" t="inlineStr">
         <is>
-          <t>+16 億 淨買</t>
+          <t>+17 億 淨買</t>
         </is>
       </c>
     </row>
@@ -4861,7 +4861,7 @@
         <v>23.08</v>
       </c>
       <c r="I6" s="212" t="n">
-        <v>-1.7</v>
+        <v>-1.71</v>
       </c>
       <c r="J6" s="71" t="inlineStr">
         <is>
@@ -6005,7 +6005,7 @@
         <v>44.44444444444444</v>
       </c>
       <c r="G42" s="208" t="n">
-        <v>1.269722222222222</v>
+        <v>1.263888888888888</v>
       </c>
     </row>
     <row r="43">
@@ -6113,7 +6113,7 @@
     <row r="4" ht="18" customHeight="1">
       <c r="B4" s="88" t="inlineStr">
         <is>
-          <t>歸因分布: 個股弱勢 (跑輸大盤 &gt;2pp): 40 | TAIEX 資料缺, 歸因不全: 38 | TAIEX 整盤跌: 15 | 假共識 (領頭獨佔 ≥50%): 9 | flat close (隔日收 = 今日收, 真實現象): 8 | alpha noise (個股無系統性原因): 3</t>
+          <t>歸因分布: 個股弱勢 (跑輸大盤 &gt;2pp): 39 | TAIEX 資料缺, 歸因不全: 38 | TAIEX 整盤跌: 15 | 假共識 (領頭獨佔 ≥50%): 9 | flat close (隔日收 = 今日收, 真實現象): 8 | alpha noise (個股無系統性原因): 4</t>
         </is>
       </c>
     </row>
@@ -6189,10 +6189,10 @@
         <v>-0.83</v>
       </c>
       <c r="F7" s="215" t="n">
-        <v>1.94</v>
+        <v>1.34</v>
       </c>
       <c r="G7" s="216" t="n">
-        <v>-2.77</v>
+        <v>-2.17</v>
       </c>
       <c r="H7" s="213" t="n">
         <v>37.3</v>
@@ -6231,10 +6231,10 @@
         <v>-3.42</v>
       </c>
       <c r="F8" s="215" t="n">
-        <v>1.94</v>
+        <v>1.34</v>
       </c>
       <c r="G8" s="216" t="n">
-        <v>-5.36</v>
+        <v>-4.76</v>
       </c>
       <c r="H8" s="213" t="n">
         <v>21.1</v>
@@ -6273,10 +6273,10 @@
         <v>-3.63</v>
       </c>
       <c r="F9" s="215" t="n">
-        <v>1.94</v>
+        <v>1.34</v>
       </c>
       <c r="G9" s="216" t="n">
-        <v>-5.57</v>
+        <v>-4.97</v>
       </c>
       <c r="H9" s="213" t="n">
         <v>21.7</v>
@@ -6315,10 +6315,10 @@
         <v>-7.46</v>
       </c>
       <c r="F10" s="215" t="n">
-        <v>1.94</v>
+        <v>1.34</v>
       </c>
       <c r="G10" s="216" t="n">
-        <v>-9.4</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="H10" s="235" t="n">
         <v>52.7</v>
@@ -6357,10 +6357,10 @@
         <v>-3.33</v>
       </c>
       <c r="F11" s="215" t="n">
-        <v>1.94</v>
+        <v>1.34</v>
       </c>
       <c r="G11" s="216" t="n">
-        <v>-5.27</v>
+        <v>-4.67</v>
       </c>
       <c r="H11" s="213" t="n">
         <v>16.8</v>
@@ -6396,13 +6396,13 @@
         </is>
       </c>
       <c r="E12" s="212" t="n">
-        <v>-6.32</v>
+        <v>-6.53</v>
       </c>
       <c r="F12" s="215" t="n">
-        <v>1.94</v>
+        <v>1.34</v>
       </c>
       <c r="G12" s="216" t="n">
-        <v>-8.26</v>
+        <v>-7.87</v>
       </c>
       <c r="H12" s="235" t="n">
         <v>67.30000000000001</v>
@@ -6441,10 +6441,10 @@
         <v>-3.6</v>
       </c>
       <c r="F13" s="215" t="n">
-        <v>1.94</v>
+        <v>1.34</v>
       </c>
       <c r="G13" s="216" t="n">
-        <v>-5.54</v>
+        <v>-4.94</v>
       </c>
       <c r="H13" s="213" t="n">
         <v>29.4</v>
@@ -6483,10 +6483,10 @@
         <v>-3.42</v>
       </c>
       <c r="F14" s="215" t="n">
-        <v>1.94</v>
+        <v>1.34</v>
       </c>
       <c r="G14" s="216" t="n">
-        <v>-5.36</v>
+        <v>-4.76</v>
       </c>
       <c r="H14" s="235" t="n">
         <v>60.09999999999999</v>
@@ -6525,10 +6525,10 @@
         <v>-0.49</v>
       </c>
       <c r="F15" s="215" t="n">
-        <v>1.94</v>
+        <v>1.34</v>
       </c>
       <c r="G15" s="216" t="n">
-        <v>-2.43</v>
+        <v>-1.83</v>
       </c>
       <c r="H15" s="213" t="n">
         <v>20.3</v>
@@ -6543,7 +6543,7 @@
       </c>
       <c r="K15" s="93" t="inlineStr">
         <is>
-          <t>個股弱勢 (跑輸大盤 &gt;2pp)</t>
+          <t>alpha noise (個股無系統性原因)</t>
         </is>
       </c>
     </row>
@@ -6567,10 +6567,10 @@
         <v>-1.32</v>
       </c>
       <c r="F16" s="215" t="n">
-        <v>1.94</v>
+        <v>1.34</v>
       </c>
       <c r="G16" s="216" t="n">
-        <v>-3.26</v>
+        <v>-2.66</v>
       </c>
       <c r="H16" s="213" t="n">
         <v>22.7</v>
@@ -18536,10 +18536,10 @@
         </is>
       </c>
       <c r="E195" s="129" t="n">
-        <v>147</v>
+        <v>271</v>
       </c>
       <c r="F195" s="129" t="n">
-        <v>40</v>
+        <v>175</v>
       </c>
       <c r="G195" s="129" t="n">
         <v>2924</v>
@@ -18551,12 +18551,12 @@
         <v>1091</v>
       </c>
       <c r="J195" s="130" t="n">
-        <v>198.93</v>
+        <v>107.91</v>
       </c>
       <c r="K195" s="130" t="n">
-        <v>458.23</v>
-      </c>
-      <c r="L195" s="220">
+        <v>104.74</v>
+      </c>
+      <c r="L195" s="219">
         <f>F195*(K195-J195)</f>
         <v/>
       </c>
@@ -18571,10 +18571,10 @@
         </is>
       </c>
       <c r="E196" s="129" t="n">
-        <v>71</v>
+        <v>204</v>
       </c>
       <c r="F196" s="129" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G196" s="129" t="n">
         <v>2793</v>
@@ -18586,12 +18586,12 @@
         <v>2181</v>
       </c>
       <c r="J196" s="130" t="n">
-        <v>393.38</v>
+        <v>136.91</v>
       </c>
       <c r="K196" s="130" t="n">
-        <v>139.11</v>
-      </c>
-      <c r="L196" s="219">
+        <v>145.74</v>
+      </c>
+      <c r="L196" s="220">
         <f>F196*(K196-J196)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-07-03 22:53
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -23,7 +23,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="24">
+  <numFmts count="25">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨+26/5d-190)&quot;;-0&quot; 億 (昨+26/5d-190)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +70億 &quot;&quot;(昨12/5d12)&quot;"/>
@@ -48,6 +48,7 @@
     <numFmt numFmtId="185" formatCode="0&quot; 檔 +90億 &quot;&quot;(昨10/5d12)&quot;"/>
     <numFmt numFmtId="186" formatCode="0.0%&quot; 市-1293億 &quot;&quot;(昨21/5d19)&quot;"/>
     <numFmt numFmtId="187" formatCode="&quot;📅 明日預測 ↑ 偏多 &quot;0.0&quot;% 信心 — 外資現貨 主推 — 3 檔焦點&quot;"/>
+    <numFmt numFmtId="188" formatCode="0.0%&quot; 市-1289億 &quot;&quot;(昨21/5d19)&quot;"/>
   </numFmts>
   <fonts count="52">
     <font>
@@ -601,7 +602,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="243">
+  <cellXfs count="244">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1165,6 +1166,9 @@
     <xf numFmtId="187" fontId="45" fillId="47" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="188" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1650,7 +1654,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 📌 一般共識 2330 / 2408 / 3711 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 除權息 8 檔: 1455, 1730, 2013 ... | 明日恐處置 9 檔: 1447/1617/3055...  |  訊號: 強偏多 (Q5 95%, hot=21)</t>
+          <t>💡 📌 一般共識 2330 / 2408 / 3711 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 除權息 8 檔: 1455, 1730, 2013 ... | 明日恐處置 3 檔: 1444/1515/1718  |  訊號: 強偏多 (Q5 95%, hot=21)</t>
         </is>
       </c>
     </row>
@@ -2384,8 +2388,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G30" s="241" t="n">
-        <v>0.2258019218974628</v>
+      <c r="G30" s="243" t="n">
+        <v>0.22600318154549</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
@@ -4829,7 +4833,7 @@
     <row r="32">
       <c r="C32" s="69" t="inlineStr">
         <is>
-          <t>明日恐處置 9 檔 (1447 / 1617 / 3055 ...)</t>
+          <t>明日恐處置 3 檔 (1444 / 1515 / 1718)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-07-03 23:42
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -2265,7 +2265,7 @@
         <v>10</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
@@ -2295,7 +2295,7 @@
         <v>7</v>
       </c>
       <c r="N25" s="18" t="n">
-        <v>16427</v>
+        <v>16143</v>
       </c>
     </row>
     <row r="26">
@@ -2316,7 +2316,7 @@
         <v>10</v>
       </c>
       <c r="F26" s="16" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
@@ -2346,7 +2346,7 @@
         <v>7</v>
       </c>
       <c r="N26" s="18" t="n">
-        <v>8968</v>
+        <v>9114</v>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
@@ -2371,7 +2371,7 @@
         </is>
       </c>
       <c r="G29" s="239" t="n">
-        <v>62.14276</v>
+        <v>62.21303</v>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
@@ -2389,7 +2389,7 @@
         </is>
       </c>
       <c r="G30" s="243" t="n">
-        <v>0.22600318154549</v>
+        <v>0.2261998468242964</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>25.9%</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2500,11 +2500,11 @@
         </is>
       </c>
       <c r="D37" s="33" t="n">
-        <v>1362450</v>
+        <v>1368762</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>24.3%</t>
+          <t>24.4%</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>張濬安(航海王)</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2724,12 +2724,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>張濬安(航海王) 今日買進 11 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 12 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>11 檔</t>
+          <t>12 檔</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="C48" s="41" t="inlineStr">
         <is>
-          <t>民哥</t>
+          <t>張濬安(航海王)</t>
         </is>
       </c>
       <c r="D48" s="41" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="E48" s="41" t="inlineStr">
         <is>
-          <t>民哥 今日買進 11 檔新標的 (過去從沒買過)</t>
+          <t>張濬安(航海王) 今日買進 11 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F48" s="41" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>民哥</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 11 檔新標的 (過去從沒買過)</t>
+          <t>民哥 今日買進 11 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -3229,77 +3229,77 @@
       </c>
     </row>
     <row r="71">
-      <c r="B71" s="35" t="inlineStr">
+      <c r="B71" s="32" t="inlineStr">
+        <is>
+          <t>陳族元</t>
+        </is>
+      </c>
+      <c r="C71" s="33" t="n">
+        <v>1315396</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>南亞科(2408)</t>
+        </is>
+      </c>
+      <c r="E71" s="33" t="n">
+        <v>159748</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>禾伸堂(3026)</t>
+        </is>
+      </c>
+      <c r="G71" s="33" t="n">
+        <v>104066</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>晶技(3042)</t>
+        </is>
+      </c>
+      <c r="I71" s="33" t="n">
+        <v>84354</v>
+      </c>
+      <c r="J71" s="202" t="n">
+        <v>0.264686903506806</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="35" t="inlineStr">
         <is>
           <t>張濬安(航海王)</t>
         </is>
       </c>
-      <c r="C71" s="33" t="n">
+      <c r="C72" s="33" t="n">
         <v>1314317</v>
       </c>
-      <c r="D71" t="inlineStr">
+      <c r="D72" t="inlineStr">
         <is>
           <t>南電(8046)</t>
         </is>
       </c>
-      <c r="E71" s="33" t="n">
+      <c r="E72" s="33" t="n">
         <v>166965</v>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F72" t="inlineStr">
         <is>
           <t>晶技(3042)</t>
         </is>
       </c>
-      <c r="G71" s="33" t="n">
+      <c r="G72" s="33" t="n">
         <v>80144</v>
       </c>
-      <c r="H71" t="inlineStr">
+      <c r="H72" t="inlineStr">
         <is>
           <t>台積電(2330)</t>
         </is>
       </c>
-      <c r="I71" s="33" t="n">
+      <c r="I72" s="33" t="n">
         <v>71983</v>
       </c>
-      <c r="J71" s="202" t="n">
+      <c r="J72" s="202" t="n">
         <v>0.2427811762045588</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" s="32" t="inlineStr">
-        <is>
-          <t>陳族元</t>
-        </is>
-      </c>
-      <c r="C72" s="33" t="n">
-        <v>1310921</v>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>南亞科(2408)</t>
-        </is>
-      </c>
-      <c r="E72" s="33" t="n">
-        <v>159748</v>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>禾伸堂(3026)</t>
-        </is>
-      </c>
-      <c r="G72" s="33" t="n">
-        <v>104066</v>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>晶技(3042)</t>
-        </is>
-      </c>
-      <c r="I72" s="33" t="n">
-        <v>84354</v>
-      </c>
-      <c r="J72" s="202" t="n">
-        <v>0.265590608615045</v>
       </c>
     </row>
     <row r="73">
@@ -18440,7 +18440,7 @@
         </is>
       </c>
       <c r="E189" s="129" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F189" s="129" t="n">
         <v>1</v>
@@ -18455,7 +18455,7 @@
         <v>6586</v>
       </c>
       <c r="J189" s="130" t="n">
-        <v>846.22</v>
+        <v>879.62</v>
       </c>
       <c r="K189" s="130" t="n">
         <v>988</v>
@@ -18475,7 +18475,7 @@
         </is>
       </c>
       <c r="E190" s="129" t="n">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F190" s="129" t="n">
         <v>54</v>
@@ -18490,12 +18490,12 @@
         <v>3487</v>
       </c>
       <c r="J190" s="130" t="n">
-        <v>400.68</v>
+        <v>409.32</v>
       </c>
       <c r="K190" s="130" t="n">
         <v>407.96</v>
       </c>
-      <c r="L190" s="220">
+      <c r="L190" s="219">
         <f>F190*(K190-J190)</f>
         <v/>
       </c>
@@ -18580,10 +18580,10 @@
         </is>
       </c>
       <c r="E193" s="129" t="n">
-        <v>137</v>
+        <v>75</v>
       </c>
       <c r="F193" s="129" t="n">
-        <v>102</v>
+        <v>54</v>
       </c>
       <c r="G193" s="129" t="n">
         <v>2522</v>
@@ -18595,12 +18595,12 @@
         <v>663</v>
       </c>
       <c r="J193" s="130" t="n">
-        <v>184.12</v>
+        <v>336.32</v>
       </c>
       <c r="K193" s="130" t="n">
-        <v>182.29</v>
-      </c>
-      <c r="L193" s="219">
+        <v>344.33</v>
+      </c>
+      <c r="L193" s="220">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -18681,29 +18681,29 @@
       <c r="C196" s="131" t="n"/>
       <c r="D196" s="128" t="inlineStr">
         <is>
-          <t>大立光(3008)</t>
+          <t>晶豪科(3006)</t>
         </is>
       </c>
       <c r="E196" s="129" t="n">
-        <v>4</v>
+        <v>94</v>
       </c>
       <c r="F196" s="129" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G196" s="129" t="n">
-        <v>1819</v>
+        <v>1988</v>
       </c>
       <c r="H196" s="129" t="n">
-        <v>0</v>
+        <v>169</v>
       </c>
       <c r="I196" s="129" t="n">
         <v>1819</v>
       </c>
       <c r="J196" s="130" t="n">
-        <v>4548.25</v>
+        <v>211.5</v>
       </c>
       <c r="K196" s="130" t="n">
-        <v>0</v>
+        <v>211.5</v>
       </c>
       <c r="L196" s="220">
         <f>F196*(K196-J196)</f>
@@ -18716,29 +18716,29 @@
       <c r="C197" s="131" t="n"/>
       <c r="D197" s="128" t="inlineStr">
         <is>
-          <t>高力(8996)</t>
+          <t>大立光(3008)</t>
         </is>
       </c>
       <c r="E197" s="129" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="F197" s="129" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G197" s="129" t="n">
-        <v>1780</v>
+        <v>1819</v>
       </c>
       <c r="H197" s="129" t="n">
-        <v>274</v>
+        <v>0</v>
       </c>
       <c r="I197" s="129" t="n">
-        <v>1506</v>
+        <v>1819</v>
       </c>
       <c r="J197" s="130" t="n">
-        <v>1369.62</v>
+        <v>4548.25</v>
       </c>
       <c r="K197" s="130" t="n">
-        <v>1370</v>
+        <v>0</v>
       </c>
       <c r="L197" s="220">
         <f>F197*(K197-J197)</f>
@@ -18751,29 +18751,29 @@
       <c r="C198" s="131" t="n"/>
       <c r="D198" s="128" t="inlineStr">
         <is>
-          <t>台半(5425)</t>
+          <t>高力(8996)</t>
         </is>
       </c>
       <c r="E198" s="129" t="n">
-        <v>105</v>
+        <v>13</v>
       </c>
       <c r="F198" s="129" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="G198" s="129" t="n">
-        <v>1352</v>
+        <v>1780</v>
       </c>
       <c r="H198" s="129" t="n">
-        <v>207</v>
+        <v>274</v>
       </c>
       <c r="I198" s="129" t="n">
-        <v>1145</v>
+        <v>1506</v>
       </c>
       <c r="J198" s="130" t="n">
-        <v>128.77</v>
+        <v>1369.62</v>
       </c>
       <c r="K198" s="130" t="n">
-        <v>129.31</v>
+        <v>1370</v>
       </c>
       <c r="L198" s="220">
         <f>F198*(K198-J198)</f>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-07-04 01:21
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -1654,7 +1654,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 📌 一般共識 2330 / 2408 / 3711 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 除權息 8 檔: 1455, 1730, 2013 ... | 明日恐處置 3 檔: 1444/1515/1718  |  訊號: 強偏多 (Q5 95%, hot=21)</t>
+          <t>💡 📌 一般共識 2330 / 2408 / 3711 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 明日恐處置 3 檔: 1444/1515/1718  |  訊號: 強偏多 (Q5 95%, hot=21)</t>
         </is>
       </c>
     </row>
@@ -2388,8 +2388,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G30" s="243" t="n">
-        <v>0.2260135027650007</v>
+      <c r="G30" s="241" t="n">
+        <v>0.2260558506983937</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
@@ -3712,7 +3712,7 @@
     <row r="85" ht="22" customHeight="1">
       <c r="B85" s="59" t="inlineStr">
         <is>
-          <t>▍ G. 注意股 (資料日 20260703)</t>
+          <t>▍ G. 注意股 (資料日 20260704)</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4112,7 @@
     <row r="107" ht="22" customHeight="1">
       <c r="B107" s="65" t="inlineStr">
         <is>
-          <t>▍ I. 未來 30 天除權息 (有效 258 檔, 已剔除過期)</t>
+          <t>▍ I. 未來 30 天除權息 (有效 266 檔, 已剔除過期)</t>
         </is>
       </c>
     </row>
@@ -4146,17 +4146,17 @@
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>20260703</t>
+          <t>20260706</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>1455</t>
+          <t>00946</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>集盛</t>
+          <t>群益科技高息成長</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -4165,23 +4165,23 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>0.16</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="110">
       <c r="B110" s="41" t="inlineStr">
         <is>
-          <t>20260703</t>
+          <t>20260706</t>
         </is>
       </c>
       <c r="C110" s="41" t="inlineStr">
         <is>
-          <t>1730</t>
+          <t>00953B</t>
         </is>
       </c>
       <c r="D110" s="41" t="inlineStr">
         <is>
-          <t>花仙子</t>
+          <t>群益優選非投等債</t>
         </is>
       </c>
       <c r="E110" s="41" t="inlineStr">
@@ -4190,23 +4190,23 @@
         </is>
       </c>
       <c r="F110" s="41" t="n">
-        <v>3</v>
+        <v>0.061</v>
       </c>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t>20260703</t>
+          <t>20260706</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>00985B</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>中鋼構</t>
+          <t>群益ESG投等債0-5</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -4215,23 +4215,23 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>2.4</v>
+        <v>0.048</v>
       </c>
     </row>
     <row r="112">
       <c r="B112" s="41" t="inlineStr">
         <is>
-          <t>20260703</t>
+          <t>20260706</t>
         </is>
       </c>
       <c r="C112" s="41" t="inlineStr">
         <is>
-          <t>2425</t>
+          <t>00997A</t>
         </is>
       </c>
       <c r="D112" s="41" t="inlineStr">
         <is>
-          <t>承啟</t>
+          <t>主動群益美國增長</t>
         </is>
       </c>
       <c r="E112" s="41" t="inlineStr">
@@ -4240,23 +4240,23 @@
         </is>
       </c>
       <c r="F112" s="41" t="n">
-        <v>0.1</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="113">
       <c r="B113" t="inlineStr">
         <is>
-          <t>20260703</t>
+          <t>20260706</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2838A</t>
+          <t>1307</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>聯邦銀甲特</t>
+          <t>三芳</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -4265,23 +4265,23 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>2.630625</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="114">
       <c r="B114" s="41" t="inlineStr">
         <is>
-          <t>20260703</t>
+          <t>20260706</t>
         </is>
       </c>
       <c r="C114" s="41" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>2373</t>
         </is>
       </c>
       <c r="D114" s="41" t="inlineStr">
         <is>
-          <t>三商家購</t>
+          <t>震旦行</t>
         </is>
       </c>
       <c r="E114" s="41" t="inlineStr">
@@ -4290,23 +4290,23 @@
         </is>
       </c>
       <c r="F114" s="41" t="n">
-        <v>1.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="115">
       <c r="B115" t="inlineStr">
         <is>
-          <t>20260703</t>
+          <t>20260706</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>3711</t>
+          <t>2474</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>日月光投控</t>
+          <t>可成</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -4315,23 +4315,23 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>6.584838</v>
+        <v>7.113868</v>
       </c>
     </row>
     <row r="116">
       <c r="B116" s="41" t="inlineStr">
         <is>
-          <t>20260703</t>
+          <t>20260706</t>
         </is>
       </c>
       <c r="C116" s="41" t="inlineStr">
         <is>
-          <t>910861</t>
+          <t>2615</t>
         </is>
       </c>
       <c r="D116" s="41" t="inlineStr">
         <is>
-          <t>神州-DR</t>
+          <t>萬海</t>
         </is>
       </c>
       <c r="E116" s="41" t="inlineStr">
@@ -4340,7 +4340,7 @@
         </is>
       </c>
       <c r="F116" s="41" t="n">
-        <v>0.072018</v>
+        <v>3</v>
       </c>
     </row>
     <row r="117">
@@ -4351,12 +4351,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>00946</t>
+          <t>2904</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>群益科技高息成長</t>
+          <t>匯僑</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -4365,7 +4365,7 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>0.058</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="118">
@@ -4376,12 +4376,12 @@
       </c>
       <c r="C118" s="41" t="inlineStr">
         <is>
-          <t>00953B</t>
+          <t>3037</t>
         </is>
       </c>
       <c r="D118" s="41" t="inlineStr">
         <is>
-          <t>群益優選非投等債</t>
+          <t>欣興</t>
         </is>
       </c>
       <c r="E118" s="41" t="inlineStr">
@@ -4390,7 +4390,7 @@
         </is>
       </c>
       <c r="F118" s="41" t="n">
-        <v>0.061</v>
+        <v>1.980153</v>
       </c>
     </row>
     <row r="119">
@@ -4401,12 +4401,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>00985B</t>
+          <t>3557</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>群益ESG投等債0-5</t>
+          <t>嘉威</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -4415,7 +4415,7 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>0.048</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="120">
@@ -4426,12 +4426,12 @@
       </c>
       <c r="C120" s="41" t="inlineStr">
         <is>
-          <t>00997A</t>
+          <t>3704</t>
         </is>
       </c>
       <c r="D120" s="41" t="inlineStr">
         <is>
-          <t>主動群益美國增長</t>
+          <t>合勤控</t>
         </is>
       </c>
       <c r="E120" s="41" t="inlineStr">
@@ -4440,7 +4440,7 @@
         </is>
       </c>
       <c r="F120" s="41" t="n">
-        <v>0.37</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="121">
@@ -4451,12 +4451,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>1307</t>
+          <t>5538</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>三芳</t>
+          <t>東明-KY</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -4465,7 +4465,7 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>2.2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="122">
@@ -4476,12 +4476,12 @@
       </c>
       <c r="C122" s="41" t="inlineStr">
         <is>
-          <t>2373</t>
+          <t>6155</t>
         </is>
       </c>
       <c r="D122" s="41" t="inlineStr">
         <is>
-          <t>震旦行</t>
+          <t>鈞寶</t>
         </is>
       </c>
       <c r="E122" s="41" t="inlineStr">
@@ -4490,7 +4490,7 @@
         </is>
       </c>
       <c r="F122" s="41" t="n">
-        <v>3.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="123">
@@ -4501,12 +4501,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2474</t>
+          <t>6754</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>可成</t>
+          <t>匯僑設計</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -4515,7 +4515,7 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>7.113868</v>
+        <v>3.5</v>
       </c>
     </row>
   </sheetData>
@@ -4824,9 +4824,9 @@
       </c>
     </row>
     <row r="31">
-      <c r="C31" s="69" t="inlineStr">
-        <is>
-          <t>除權息 8 檔 (1455 / 1730 / 2013 ...)</t>
+      <c r="C31" s="71" t="inlineStr">
+        <is>
+          <t>今日無除權息</t>
         </is>
       </c>
     </row>
@@ -10880,7 +10880,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="B3" s="98" t="inlineStr">
         <is>
-          <t>大牌分析師 近 52/52 交易日出手 2511 次 (529 檔), 風格分布: 隔日沖近似 39% / 當沖 13% / 留倉 48%, 漲停命中 5% (其中 🔒鎖漲停 4%), 前 5 大集中 25%, 長線部位 63% (37 檔), ⚠️ 處置股部位 11% (43 檔), 📦 連續囤貨 29 檔 (最長 13 天 009816, 2 檔仍 active)。 主軸: 高頻交易/持續進場/📦 連續囤貨。</t>
+          <t>大牌分析師 近 52/52 交易日出手 2511 次 (529 檔), 風格分布: 隔日沖近似 39% / 當沖 13% / 留倉 48%, 漲停命中 5% (其中 🔒鎖漲停 4%), 前 5 大集中 25%, 長線部位 63% (37 檔), ⚠️ 處置股部位 12% (35 檔), 📦 連續囤貨 29 檔 (最長 13 天 009816, 2 檔仍 active)。 主軸: 高頻交易/持續進場/📦 連續囤貨。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-07-06 10:46
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -1687,9 +1687,9 @@
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>🔬 Phase 3.5 多日 alpha (觀察期 n=38): 5 日內擇高 86.8% / +12.78%  |  premium 擇高 92.9% / +15.99% (n=28)  |  premium 持有 3 天 92.9% / +12.16%  — 來源: quad_hit_log × stock_history t+1~t+5</t>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>🚀 Phase 3.5 多日 alpha (正式): 5 日內擇高 72.8% / +8.56%  |  premium 擇高 73.5% / +9.61% (n=83)  |  premium 持有 3 天 75.7% / +6.37%  — 來源: quad_hit_log × stock_history t+1~t+5</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1710,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>📌 大牌分析師 歷史 alpha: 全 picks n=1461 hit_1d=48% / hit_3d=51%  |  新標 n=302 hit_3d=49% mean=+0.96%  |  連加 n=69 hit_5d=59% mean=+3.86%</t>
+          <t>📌 大牌分析師 歷史 alpha: 全 picks n=1641 hit_1d=49% / hit_3d=51%  |  新標 n=314 hit_3d=50% mean=+1.07%  |  連加 n=80 hit_5d=57% mean=+3.63%</t>
         </is>
       </c>
     </row>
@@ -2265,7 +2265,7 @@
         <v>10</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
@@ -2295,7 +2295,7 @@
         <v>7</v>
       </c>
       <c r="N25" s="18" t="n">
-        <v>16143</v>
+        <v>16427</v>
       </c>
     </row>
     <row r="26">
@@ -2316,7 +2316,7 @@
         <v>10</v>
       </c>
       <c r="F26" s="16" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
@@ -2346,7 +2346,7 @@
         <v>7</v>
       </c>
       <c r="N26" s="18" t="n">
-        <v>9114</v>
+        <v>8968</v>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
@@ -2371,7 +2371,7 @@
         </is>
       </c>
       <c r="G29" s="239" t="n">
-        <v>62.21303</v>
+        <v>62.13752</v>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
@@ -2389,7 +2389,7 @@
         </is>
       </c>
       <c r="G30" s="241" t="n">
-        <v>0.2260558506983937</v>
+        <v>0.2258069783531962</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
@@ -2400,7 +2400,7 @@
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="28" t="inlineStr">
         <is>
-          <t>✅ 過去 30 天 P/C 命中率: 偏多 18/27 (67%) | 偏空 0/0 (0%) | 整體 18/27 (67%)</t>
+          <t>✅ 過去 30 天 P/C 命中率: 偏多 19/28 (68%) | 偏空 0/0 (0%) | 整體 19/28 (68%)</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>25.9%</t>
+          <t>26.0%</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2500,11 +2500,11 @@
         </is>
       </c>
       <c r="D37" s="33" t="n">
-        <v>1368762</v>
+        <v>1362450</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>24.3%</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>張濬安(航海王)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2724,12 +2724,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 12 檔新標的 (過去從沒買過)</t>
+          <t>張濬安(航海王) 今日買進 11 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>12 檔</t>
+          <t>11 檔</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="C48" s="41" t="inlineStr">
         <is>
-          <t>張濬安(航海王)</t>
+          <t>民哥</t>
         </is>
       </c>
       <c r="D48" s="41" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="E48" s="41" t="inlineStr">
         <is>
-          <t>張濬安(航海王) 今日買進 11 檔新標的 (過去從沒買過)</t>
+          <t>民哥 今日買進 11 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F48" s="41" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>民哥</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>民哥 今日買進 11 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 11 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2832,12 +2832,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>大牌分析師 今日買進 8 檔新標的 (過去從沒買過)</t>
+          <t>大牌分析師 今日買進 9 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>8 檔</t>
+          <t>9 檔</t>
         </is>
       </c>
     </row>
@@ -3229,77 +3229,77 @@
       </c>
     </row>
     <row r="71">
-      <c r="B71" s="32" t="inlineStr">
+      <c r="B71" s="35" t="inlineStr">
+        <is>
+          <t>張濬安(航海王)</t>
+        </is>
+      </c>
+      <c r="C71" s="33" t="n">
+        <v>1314317</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>南電(8046)</t>
+        </is>
+      </c>
+      <c r="E71" s="33" t="n">
+        <v>166965</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>晶技(3042)</t>
+        </is>
+      </c>
+      <c r="G71" s="33" t="n">
+        <v>80144</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>台積電(2330)</t>
+        </is>
+      </c>
+      <c r="I71" s="33" t="n">
+        <v>71983</v>
+      </c>
+      <c r="J71" s="202" t="n">
+        <v>0.2427811762045588</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="32" t="inlineStr">
         <is>
           <t>陳族元</t>
         </is>
       </c>
-      <c r="C71" s="33" t="n">
-        <v>1315396</v>
-      </c>
-      <c r="D71" t="inlineStr">
+      <c r="C72" s="33" t="n">
+        <v>1310921</v>
+      </c>
+      <c r="D72" t="inlineStr">
         <is>
           <t>南亞科(2408)</t>
         </is>
       </c>
-      <c r="E71" s="33" t="n">
+      <c r="E72" s="33" t="n">
         <v>159748</v>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F72" t="inlineStr">
         <is>
           <t>禾伸堂(3026)</t>
         </is>
       </c>
-      <c r="G71" s="33" t="n">
+      <c r="G72" s="33" t="n">
         <v>104066</v>
       </c>
-      <c r="H71" t="inlineStr">
+      <c r="H72" t="inlineStr">
         <is>
           <t>晶技(3042)</t>
         </is>
       </c>
-      <c r="I71" s="33" t="n">
+      <c r="I72" s="33" t="n">
         <v>84354</v>
       </c>
-      <c r="J71" s="202" t="n">
-        <v>0.264686903506806</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" s="35" t="inlineStr">
-        <is>
-          <t>張濬安(航海王)</t>
-        </is>
-      </c>
-      <c r="C72" s="33" t="n">
-        <v>1314317</v>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>南電(8046)</t>
-        </is>
-      </c>
-      <c r="E72" s="33" t="n">
-        <v>166965</v>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>晶技(3042)</t>
-        </is>
-      </c>
-      <c r="G72" s="33" t="n">
-        <v>80144</v>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>台積電(2330)</t>
-        </is>
-      </c>
-      <c r="I72" s="33" t="n">
-        <v>71983</v>
-      </c>
       <c r="J72" s="202" t="n">
-        <v>0.2427811762045588</v>
+        <v>0.265590608615045</v>
       </c>
     </row>
     <row r="73">
@@ -3642,7 +3642,7 @@
         </is>
       </c>
       <c r="C82" s="33" t="n">
-        <v>77663</v>
+        <v>77863</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3669,7 +3669,7 @@
         <v>5947</v>
       </c>
       <c r="J82" s="202" t="n">
-        <v>0.3001381612069598</v>
+        <v>0.2993652987154427</v>
       </c>
     </row>
     <row r="83">
@@ -3712,7 +3712,7 @@
     <row r="85" ht="22" customHeight="1">
       <c r="B85" s="59" t="inlineStr">
         <is>
-          <t>▍ G. 注意股 (資料日 20260704)</t>
+          <t>▍ G. 注意股 (資料日 20260706)</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4112,7 @@
     <row r="107" ht="22" customHeight="1">
       <c r="B107" s="65" t="inlineStr">
         <is>
-          <t>▍ I. 未來 30 天除權息 (有效 266 檔, 已剔除過期)</t>
+          <t>▍ I. 未來 30 天除權息 (有效 270 檔, 已剔除過期)</t>
         </is>
       </c>
     </row>
@@ -10888,21 +10888,21 @@
     <row r="6">
       <c r="B6" s="99" t="inlineStr">
         <is>
-          <t>全部 picks: n=1461  hit_1d=48%  mean_1d=+0.21%  hit_3d=51%  mean_3d=+0.78%  hit_5d=54%  mean_5d=+2.17%</t>
+          <t>全部 picks: n=1641  hit_1d=49%  mean_1d=+0.26%  hit_3d=51%  mean_3d=+0.86%  hit_5d=52%  mean_5d=+1.91%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="99" t="inlineStr">
         <is>
-          <t>新標的: n=302  hit_1d=48%  mean_1d=+0.25%  hit_3d=49%  mean_3d=+0.96%  hit_5d=52%  mean_5d=+2.36%</t>
+          <t>新標的: n=314  hit_1d=48%  mean_1d=+0.21%  hit_3d=50%  mean_3d=+1.07%  hit_5d=52%  mean_5d=+2.33%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="99" t="inlineStr">
         <is>
-          <t>連續加碼: n=69  hit_1d=48%  mean_1d=+0.87%  hit_3d=52%  mean_3d=-3.16%  hit_5d=59%  mean_5d=+3.86%</t>
+          <t>連續加碼: n=80  hit_1d=52%  mean_1d=+1.16%  hit_3d=53%  mean_3d=-2.53%  hit_5d=57%  mean_5d=+3.63%</t>
         </is>
       </c>
     </row>
@@ -11038,7 +11038,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="201" t="n">
-        <v>-0.0528</v>
+        <v>-0.0619</v>
       </c>
     </row>
     <row r="16">
@@ -18440,7 +18440,7 @@
         </is>
       </c>
       <c r="E189" s="129" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F189" s="129" t="n">
         <v>1</v>
@@ -18455,7 +18455,7 @@
         <v>6586</v>
       </c>
       <c r="J189" s="130" t="n">
-        <v>879.62</v>
+        <v>846.22</v>
       </c>
       <c r="K189" s="130" t="n">
         <v>988</v>
@@ -18475,7 +18475,7 @@
         </is>
       </c>
       <c r="E190" s="129" t="n">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F190" s="129" t="n">
         <v>54</v>
@@ -18490,12 +18490,12 @@
         <v>3487</v>
       </c>
       <c r="J190" s="130" t="n">
-        <v>409.32</v>
+        <v>400.68</v>
       </c>
       <c r="K190" s="130" t="n">
         <v>407.96</v>
       </c>
-      <c r="L190" s="219">
+      <c r="L190" s="220">
         <f>F190*(K190-J190)</f>
         <v/>
       </c>
@@ -18580,10 +18580,10 @@
         </is>
       </c>
       <c r="E193" s="129" t="n">
-        <v>75</v>
+        <v>137</v>
       </c>
       <c r="F193" s="129" t="n">
-        <v>54</v>
+        <v>102</v>
       </c>
       <c r="G193" s="129" t="n">
         <v>2522</v>
@@ -18595,12 +18595,12 @@
         <v>663</v>
       </c>
       <c r="J193" s="130" t="n">
-        <v>336.32</v>
+        <v>184.12</v>
       </c>
       <c r="K193" s="130" t="n">
-        <v>344.33</v>
-      </c>
-      <c r="L193" s="220">
+        <v>182.29</v>
+      </c>
+      <c r="L193" s="219">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -18681,29 +18681,29 @@
       <c r="C196" s="131" t="n"/>
       <c r="D196" s="128" t="inlineStr">
         <is>
-          <t>晶豪科(3006)</t>
+          <t>大立光(3008)</t>
         </is>
       </c>
       <c r="E196" s="129" t="n">
-        <v>94</v>
+        <v>4</v>
       </c>
       <c r="F196" s="129" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G196" s="129" t="n">
-        <v>1988</v>
+        <v>1819</v>
       </c>
       <c r="H196" s="129" t="n">
-        <v>169</v>
+        <v>0</v>
       </c>
       <c r="I196" s="129" t="n">
         <v>1819</v>
       </c>
       <c r="J196" s="130" t="n">
-        <v>211.5</v>
+        <v>4548.25</v>
       </c>
       <c r="K196" s="130" t="n">
-        <v>211.5</v>
+        <v>0</v>
       </c>
       <c r="L196" s="220">
         <f>F196*(K196-J196)</f>
@@ -18716,29 +18716,29 @@
       <c r="C197" s="131" t="n"/>
       <c r="D197" s="128" t="inlineStr">
         <is>
-          <t>大立光(3008)</t>
+          <t>高力(8996)</t>
         </is>
       </c>
       <c r="E197" s="129" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F197" s="129" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G197" s="129" t="n">
-        <v>1819</v>
+        <v>1780</v>
       </c>
       <c r="H197" s="129" t="n">
-        <v>0</v>
+        <v>274</v>
       </c>
       <c r="I197" s="129" t="n">
-        <v>1819</v>
+        <v>1506</v>
       </c>
       <c r="J197" s="130" t="n">
-        <v>4548.25</v>
+        <v>1369.62</v>
       </c>
       <c r="K197" s="130" t="n">
-        <v>0</v>
+        <v>1370</v>
       </c>
       <c r="L197" s="220">
         <f>F197*(K197-J197)</f>
@@ -18751,29 +18751,29 @@
       <c r="C198" s="131" t="n"/>
       <c r="D198" s="128" t="inlineStr">
         <is>
-          <t>高力(8996)</t>
+          <t>台半(5425)</t>
         </is>
       </c>
       <c r="E198" s="129" t="n">
-        <v>13</v>
+        <v>105</v>
       </c>
       <c r="F198" s="129" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="G198" s="129" t="n">
-        <v>1780</v>
+        <v>1352</v>
       </c>
       <c r="H198" s="129" t="n">
-        <v>274</v>
+        <v>207</v>
       </c>
       <c r="I198" s="129" t="n">
-        <v>1506</v>
+        <v>1145</v>
       </c>
       <c r="J198" s="130" t="n">
-        <v>1369.62</v>
+        <v>128.77</v>
       </c>
       <c r="K198" s="130" t="n">
-        <v>1370</v>
+        <v>129.31</v>
       </c>
       <c r="L198" s="220">
         <f>F198*(K198-J198)</f>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-07-06 22:53
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -1605,7 +1605,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 📌 一般共識 2330 / 2383 / 2308 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 除權息 22 檔: 00946, 00953B, 00985B ... | 明日恐處置 3 檔: 1444/1515/1718  |  訊號: 強偏多 (Q5 95%, hot=19)</t>
+          <t>💡 📌 一般共識 2330 / 2383 / 2308 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 除權息 22 檔: 00946, 00953B, 00985B ... | 明日恐處置 8 檔: 2466/3026/3167...  |  訊號: 強偏多 (Q5 95%, hot=19)</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2595,7 @@
         </is>
       </c>
       <c r="G35" s="246" t="n">
-        <v>0.1877375185157214</v>
+        <v>0.1880521603928755</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
@@ -5035,7 +5035,7 @@
     <row r="31">
       <c r="C31" s="69" t="inlineStr">
         <is>
-          <t>明日恐處置 3 檔 (1444 / 1515 / 1718)</t>
+          <t>明日恐處置 8 檔 (2466 / 3026 / 3167 ...)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-07-07 01:45
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -24,7 +24,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="28">
+  <numFmts count="29">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨+26/5d-190)&quot;;-0&quot; 億 (昨+26/5d-190)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +70億 &quot;&quot;(昨12/5d12)&quot;"/>
@@ -53,6 +53,7 @@
     <numFmt numFmtId="189" formatCode="+0&quot; 億 (昨+62/5d-34)&quot;;-0&quot; 億 (昨+62/5d-34)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="190" formatCode="0&quot; 檔 +75億 &quot;&quot;(昨11/5d12)&quot;"/>
     <numFmt numFmtId="191" formatCode="0.0%&quot; 市-1269億 &quot;&quot;(昨23/5d20)&quot;"/>
+    <numFmt numFmtId="192" formatCode="0.0%&quot; 市-1270億 &quot;&quot;(昨23/5d20)&quot;"/>
   </numFmts>
   <fonts count="52">
     <font>
@@ -606,7 +607,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="247">
+  <cellXfs count="248">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1182,6 +1183,9 @@
     <xf numFmtId="191" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="192" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2594,8 +2598,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G35" s="246" t="n">
-        <v>0.1877375185157214</v>
+      <c r="G35" s="247" t="n">
+        <v>0.187868889492441</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-07-07 02:17
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -24,7 +24,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="29">
+  <numFmts count="30">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨+26/5d-190)&quot;;-0&quot; 億 (昨+26/5d-190)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +70億 &quot;&quot;(昨12/5d12)&quot;"/>
@@ -54,6 +54,7 @@
     <numFmt numFmtId="190" formatCode="0&quot; 檔 +75億 &quot;&quot;(昨11/5d12)&quot;"/>
     <numFmt numFmtId="191" formatCode="0.0%&quot; 市-1269億 &quot;&quot;(昨23/5d20)&quot;"/>
     <numFmt numFmtId="192" formatCode="0.0%&quot; 市-1270億 &quot;&quot;(昨23/5d20)&quot;"/>
+    <numFmt numFmtId="193" formatCode="0.0%&quot; 市-1274億 &quot;&quot;(昨23/5d20)&quot;"/>
   </numFmts>
   <fonts count="52">
     <font>
@@ -607,7 +608,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="248">
+  <cellXfs count="249">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1186,6 +1187,9 @@
     <xf numFmtId="192" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="193" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2581,7 +2585,7 @@
         </is>
       </c>
       <c r="G34" s="244" t="n">
-        <v>-173.9864</v>
+        <v>-173.97844</v>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
@@ -2598,8 +2602,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G35" s="247" t="n">
-        <v>0.187868889492441</v>
+      <c r="G35" s="248" t="n">
+        <v>0.1881211267889168</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
@@ -2678,7 +2682,7 @@
         </is>
       </c>
       <c r="D41" s="33" t="n">
-        <v>1154176</v>
+        <v>1153606</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2742,7 +2746,7 @@
         </is>
       </c>
       <c r="D43" s="33" t="n">
-        <v>460978</v>
+        <v>460109</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2806,7 +2810,7 @@
         </is>
       </c>
       <c r="D45" s="33" t="n">
-        <v>318848</v>
+        <v>318384</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2897,7 +2901,7 @@
       </c>
       <c r="C51" s="41" t="inlineStr">
         <is>
-          <t>張濬安(航海王)</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="D51" s="41" t="inlineStr">
@@ -2907,7 +2911,7 @@
       </c>
       <c r="E51" s="41" t="inlineStr">
         <is>
-          <t>張濬安(航海王) 今日買進 12 檔新標的 (過去從沒買過)</t>
+          <t>林滄海 今日買進 12 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F51" s="41" t="inlineStr">
@@ -2924,7 +2928,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>林滄海</t>
+          <t>張濬安(航海王)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2934,12 +2938,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>林滄海 今日買進 12 檔新標的 (過去從沒買過)</t>
+          <t>張濬安(航海王) 今日買進 11 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>12 檔</t>
+          <t>11 檔</t>
         </is>
       </c>
     </row>
@@ -2961,12 +2965,12 @@
       </c>
       <c r="E53" s="41" t="inlineStr">
         <is>
-          <t>迷你哥/松山哥 今日買進 9 檔新標的 (過去從沒買過)</t>
+          <t>迷你哥/松山哥 今日買進 8 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F53" s="41" t="inlineStr">
         <is>
-          <t>9 檔</t>
+          <t>8 檔</t>
         </is>
       </c>
     </row>
@@ -3445,7 +3449,7 @@
         </is>
       </c>
       <c r="C76" s="33" t="n">
-        <v>1044072</v>
+        <v>1043502</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3472,7 +3476,7 @@
         <v>42623</v>
       </c>
       <c r="J76" s="202" t="n">
-        <v>0.2477659349387844</v>
+        <v>0.2479012739888113</v>
       </c>
     </row>
     <row r="77">
@@ -3519,7 +3523,7 @@
         </is>
       </c>
       <c r="C78" s="33" t="n">
-        <v>458228</v>
+        <v>457359</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3546,7 +3550,7 @@
         <v>38253</v>
       </c>
       <c r="J78" s="202" t="n">
-        <v>0.3982710350024518</v>
+        <v>0.3990277657218434</v>
       </c>
     </row>
     <row r="79">
@@ -3593,7 +3597,7 @@
         </is>
       </c>
       <c r="C80" s="33" t="n">
-        <v>294519</v>
+        <v>294055</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3620,7 +3624,7 @@
         <v>15058</v>
       </c>
       <c r="J80" s="202" t="n">
-        <v>0.2139676415094019</v>
+        <v>0.2143051955515865</v>
       </c>
     </row>
     <row r="81">
@@ -3630,7 +3634,7 @@
         </is>
       </c>
       <c r="C81" s="33" t="n">
-        <v>235161</v>
+        <v>234766</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3657,7 +3661,7 @@
         <v>14181</v>
       </c>
       <c r="J81" s="202" t="n">
-        <v>0.1833723208237424</v>
+        <v>0.183680380292759</v>
       </c>
     </row>
     <row r="82">
@@ -3667,7 +3671,7 @@
         </is>
       </c>
       <c r="C82" s="33" t="n">
-        <v>175971</v>
+        <v>175726</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3694,7 +3698,7 @@
         <v>13013</v>
       </c>
       <c r="J82" s="202" t="n">
-        <v>0.2923942976838176</v>
+        <v>0.292801959418548</v>
       </c>
     </row>
     <row r="83">
@@ -3704,7 +3708,7 @@
         </is>
       </c>
       <c r="C83" s="33" t="n">
-        <v>155253</v>
+        <v>155270</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3731,7 +3735,7 @@
         <v>9585</v>
       </c>
       <c r="J83" s="202" t="n">
-        <v>0.2588144891335363</v>
+        <v>0.2587864857084157</v>
       </c>
     </row>
     <row r="84">
@@ -3815,7 +3819,7 @@
         </is>
       </c>
       <c r="C86" s="33" t="n">
-        <v>75692</v>
+        <v>75091</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3842,7 +3846,7 @@
         <v>5286</v>
       </c>
       <c r="J86" s="202" t="n">
-        <v>0.2571593149041637</v>
+        <v>0.2592158058678059</v>
       </c>
     </row>
     <row r="87">
@@ -3852,7 +3856,7 @@
         </is>
       </c>
       <c r="C87" s="33" t="n">
-        <v>71734</v>
+        <v>71669</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3879,7 +3883,7 @@
         <v>5158</v>
       </c>
       <c r="J87" s="202" t="n">
-        <v>0.2255496339955474</v>
+        <v>0.225753565334111</v>
       </c>
     </row>
     <row r="88">
@@ -3889,7 +3893,7 @@
         </is>
       </c>
       <c r="C88" s="33" t="n">
-        <v>35719</v>
+        <v>35546</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3916,7 +3920,7 @@
         <v>2724</v>
       </c>
       <c r="J88" s="202" t="n">
-        <v>0.3575563979238173</v>
+        <v>0.3593006245428459</v>
       </c>
     </row>
     <row r="90" ht="22" customHeight="1">
@@ -27263,31 +27267,31 @@
       <c r="C416" s="178" t="n"/>
       <c r="D416" s="175" t="inlineStr">
         <is>
-          <t>菱生(2369)</t>
+          <t>聯傑(3094)</t>
         </is>
       </c>
       <c r="E416" s="176" t="n">
-        <v>1893</v>
+        <v>1475</v>
       </c>
       <c r="F416" s="176" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="G416" s="176" t="n">
-        <v>8177</v>
+        <v>6328</v>
       </c>
       <c r="H416" s="176" t="n">
-        <v>115</v>
+        <v>4</v>
       </c>
       <c r="I416" s="176" t="n">
-        <v>8062</v>
+        <v>6324</v>
       </c>
       <c r="J416" s="177" t="n">
-        <v>43.2</v>
+        <v>42.9</v>
       </c>
       <c r="K416" s="177" t="n">
-        <v>42.74</v>
-      </c>
-      <c r="L416" s="219">
+        <v>43</v>
+      </c>
+      <c r="L416" s="220">
         <f>F416*(K416-J416)</f>
         <v/>
       </c>
@@ -27298,29 +27302,29 @@
       <c r="C417" s="178" t="n"/>
       <c r="D417" s="175" t="inlineStr">
         <is>
-          <t>聯傑(3094)</t>
+          <t>大亞(1609)</t>
         </is>
       </c>
       <c r="E417" s="176" t="n">
-        <v>1475</v>
+        <v>1012</v>
       </c>
       <c r="F417" s="176" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G417" s="176" t="n">
-        <v>6328</v>
+        <v>4427</v>
       </c>
       <c r="H417" s="176" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="I417" s="176" t="n">
-        <v>6324</v>
+        <v>4395</v>
       </c>
       <c r="J417" s="177" t="n">
-        <v>42.9</v>
+        <v>43.75</v>
       </c>
       <c r="K417" s="177" t="n">
-        <v>43</v>
+        <v>45.86</v>
       </c>
       <c r="L417" s="220">
         <f>F417*(K417-J417)</f>
@@ -27333,31 +27337,31 @@
       <c r="C418" s="178" t="n"/>
       <c r="D418" s="175" t="inlineStr">
         <is>
-          <t>大亞(1609)</t>
+          <t>長榮航太(2645)</t>
         </is>
       </c>
       <c r="E418" s="176" t="n">
-        <v>1012</v>
+        <v>63</v>
       </c>
       <c r="F418" s="176" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="G418" s="176" t="n">
-        <v>4427</v>
+        <v>1489</v>
       </c>
       <c r="H418" s="176" t="n">
-        <v>32</v>
+        <v>635</v>
       </c>
       <c r="I418" s="176" t="n">
-        <v>4395</v>
+        <v>854</v>
       </c>
       <c r="J418" s="177" t="n">
-        <v>43.75</v>
+        <v>236.33</v>
       </c>
       <c r="K418" s="177" t="n">
-        <v>45.86</v>
-      </c>
-      <c r="L418" s="220">
+        <v>235.3</v>
+      </c>
+      <c r="L418" s="219">
         <f>F418*(K418-J418)</f>
         <v/>
       </c>
@@ -27609,29 +27613,29 @@
       <c r="C425" s="178" t="n"/>
       <c r="D425" s="175" t="inlineStr">
         <is>
-          <t>映泰(2399)</t>
+          <t>廣閎科(6693)</t>
         </is>
       </c>
       <c r="E425" s="176" t="n">
-        <v>158</v>
+        <v>30</v>
       </c>
       <c r="F425" s="176" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="G425" s="176" t="n">
-        <v>869</v>
+        <v>836</v>
       </c>
       <c r="H425" s="176" t="n">
-        <v>148</v>
+        <v>0</v>
       </c>
       <c r="I425" s="176" t="n">
-        <v>721</v>
+        <v>836</v>
       </c>
       <c r="J425" s="177" t="n">
-        <v>55</v>
+        <v>278.8</v>
       </c>
       <c r="K425" s="177" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="L425" s="220">
         <f>F425*(K425-J425)</f>
@@ -27642,46 +27646,25 @@
       <c r="A426" s="178" t="n"/>
       <c r="B426" s="178" t="n"/>
       <c r="C426" s="178" t="n"/>
-      <c r="D426" s="175" t="inlineStr">
-        <is>
-          <t>廣閎科(6693)</t>
-        </is>
-      </c>
-      <c r="E426" s="176" t="n">
-        <v>30</v>
-      </c>
-      <c r="F426" s="176" t="n">
-        <v>0</v>
-      </c>
-      <c r="G426" s="176" t="n">
-        <v>836</v>
-      </c>
-      <c r="H426" s="176" t="n">
-        <v>0</v>
-      </c>
-      <c r="I426" s="176" t="n">
-        <v>836</v>
-      </c>
-      <c r="J426" s="177" t="n">
-        <v>278.8</v>
-      </c>
-      <c r="K426" s="177" t="n">
-        <v>0</v>
-      </c>
-      <c r="L426" s="220">
-        <f>F426*(K426-J426)</f>
-        <v/>
-      </c>
+      <c r="D426" s="180" t="inlineStr">
+        <is>
+          <t>⚪ 今日漲停僅 6 檔</t>
+        </is>
+      </c>
+      <c r="E426" s="176" t="n"/>
+      <c r="F426" s="176" t="n"/>
+      <c r="G426" s="176" t="n"/>
+      <c r="H426" s="176" t="n"/>
+      <c r="I426" s="176" t="n"/>
+      <c r="J426" s="177" t="n"/>
+      <c r="K426" s="177" t="n"/>
+      <c r="L426" s="221" t="n"/>
     </row>
     <row r="427" ht="16.5" customHeight="1">
       <c r="A427" s="178" t="n"/>
       <c r="B427" s="178" t="n"/>
       <c r="C427" s="178" t="n"/>
-      <c r="D427" s="180" t="inlineStr">
-        <is>
-          <t>⚪ 今日漲停僅 7 檔</t>
-        </is>
-      </c>
+      <c r="D427" s="175" t="n"/>
       <c r="E427" s="176" t="n"/>
       <c r="F427" s="176" t="n"/>
       <c r="G427" s="176" t="n"/>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-07-07 11:18
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-07.xlsx
+++ b/data/reports/chip_radar_2026-07.xlsx
@@ -1613,7 +1613,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 📌 一般共識 2330 / 2383 / 2308 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 除權息 22 檔: 00946, 00953B, 00985B ... | 明日恐處置 8 檔: 2466/3026/3167...  |  訊號: 強偏多 (Q5 95%, hot=19)</t>
+          <t>💡 📌 一般共識 2330 / 2383 / 2308 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 明日恐處置 8 檔: 2466/3026/3167...  |  訊號: 強偏多 (Q5 95%, hot=19)</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2585,7 @@
         </is>
       </c>
       <c r="G34" s="244" t="n">
-        <v>-173.97844</v>
+        <v>-173.99525</v>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
@@ -2602,8 +2602,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G35" s="248" t="n">
-        <v>0.1881211267889168</v>
+      <c r="G35" s="247" t="n">
+        <v>0.1877312504931147</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
@@ -2614,7 +2614,7 @@
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="28" t="inlineStr">
         <is>
-          <t>✅ 過去 30 天 P/C 命中率: 偏多 18/27 (67%) | 偏空 0/0 (0%) | 整體 18/27 (67%)</t>
+          <t>✅ 過去 30 天 P/C 命中率: 偏多 18/28 (64%) | 偏空 0/0 (0%) | 整體 18/28 (64%)</t>
         </is>
       </c>
     </row>
@@ -2682,7 +2682,7 @@
         </is>
       </c>
       <c r="D41" s="33" t="n">
-        <v>1153606</v>
+        <v>1154176</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2746,7 +2746,7 @@
         </is>
       </c>
       <c r="D43" s="33" t="n">
-        <v>460109</v>
+        <v>460978</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2810,7 +2810,7 @@
         </is>
       </c>
       <c r="D45" s="33" t="n">
-        <v>318384</v>
+        <v>318848</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="C51" s="41" t="inlineStr">
         <is>
-          <t>林滄海</t>
+          <t>張濬安(航海王)</t>
         </is>
       </c>
       <c r="D51" s="41" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="E51" s="41" t="inlineStr">
         <is>
-          <t>林滄海 今日買進 12 檔新標的 (過去從沒買過)</t>
+          <t>張濬安(航海王) 今日買進 12 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F51" s="41" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>張濬安(航海王)</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2938,12 +2938,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>張濬安(航海王) 今日買進 11 檔新標的 (過去從沒買過)</t>
+          <t>林滄海 今日買進 12 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>11 檔</t>
+          <t>12 檔</t>
         </is>
       </c>
     </row>
@@ -2965,12 +2965,12 @@
       </c>
       <c r="E53" s="41" t="inlineStr">
         <is>
-          <t>迷你哥/松山哥 今日買進 8 檔新標的 (過去從沒買過)</t>
+          <t>迷你哥/松山哥 今日買進 9 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F53" s="41" t="inlineStr">
         <is>
-          <t>8 檔</t>
+          <t>9 檔</t>
         </is>
       </c>
     </row>
@@ -2982,7 +2982,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Tradow</t>
+          <t>民哥</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2992,12 +2992,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Tradow 今日買進 7 檔新標的 (過去從沒買過)</t>
+          <t>民哥 今日買進 8 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>7 檔</t>
+          <t>8 檔</t>
         </is>
       </c>
     </row>
@@ -3009,7 +3009,7 @@
       </c>
       <c r="C55" s="41" t="inlineStr">
         <is>
-          <t>巨人傑</t>
+          <t>Tradow</t>
         </is>
       </c>
       <c r="D55" s="41" t="inlineStr">
@@ -3019,7 +3019,7 @@
       </c>
       <c r="E55" s="41" t="inlineStr">
         <is>
-          <t>巨人傑 今日買進 7 檔新標的 (過去從沒買過)</t>
+          <t>Tradow 今日買進 7 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F55" s="41" t="inlineStr">
@@ -3036,7 +3036,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>民哥</t>
+          <t>巨人傑</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>民哥 今日買進 7 檔新標的 (過去從沒買過)</t>
+          <t>巨人傑 今日買進 7 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3073,12 +3073,12 @@
       </c>
       <c r="E57" s="41" t="inlineStr">
         <is>
-          <t>強森 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>強森 今日買進 7 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F57" s="41" t="inlineStr">
         <is>
-          <t>6 檔</t>
+          <t>7 檔</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3449,7 @@
         </is>
       </c>
       <c r="C76" s="33" t="n">
-        <v>1043502</v>
+        <v>1044072</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3476,7 +3476,7 @@
         <v>42623</v>
       </c>
       <c r="J76" s="202" t="n">
-        <v>0.2479012739888113</v>
+        <v>0.2477659349387844</v>
       </c>
     </row>
     <row r="77">
@@ -3523,7 +3523,7 @@
         </is>
       </c>
       <c r="C78" s="33" t="n">
-        <v>457359</v>
+        <v>458228</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3550,7 +3550,7 @@
         <v>38253</v>
       </c>
       <c r="J78" s="202" t="n">
-        <v>0.3990277657218434</v>
+        <v>0.3982710350024518</v>
       </c>
     </row>
     <row r="79">
@@ -3597,7 +3597,7 @@
         </is>
       </c>
       <c r="C80" s="33" t="n">
-        <v>294055</v>
+        <v>294519</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3624,7 +3624,7 @@
         <v>15058</v>
       </c>
       <c r="J80" s="202" t="n">
-        <v>0.2143051955515865</v>
+        <v>0.2139676415094019</v>
       </c>
     </row>
     <row r="81">
@@ -3634,7 +3634,7 @@
         </is>
       </c>
       <c r="C81" s="33" t="n">
-        <v>234766</v>
+        <v>235161</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3661,7 +3661,7 @@
         <v>14181</v>
       </c>
       <c r="J81" s="202" t="n">
-        <v>0.183680380292759</v>
+        <v>0.1833723208237424</v>
       </c>
     </row>
     <row r="82">
@@ -3671,7 +3671,7 @@
         </is>
       </c>
       <c r="C82" s="33" t="n">
-        <v>175726</v>
+        <v>175971</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3698,7 +3698,7 @@
         <v>13013</v>
       </c>
       <c r="J82" s="202" t="n">
-        <v>0.292801959418548</v>
+        <v>0.2923942976838176</v>
       </c>
     </row>
     <row r="83">
@@ -3708,7 +3708,7 @@
         </is>
       </c>
       <c r="C83" s="33" t="n">
-        <v>155270</v>
+        <v>155290</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3735,7 +3735,7 @@
         <v>9585</v>
       </c>
       <c r="J83" s="202" t="n">
-        <v>0.2587864857084157</v>
+        <v>0.2587519898203623</v>
       </c>
     </row>
     <row r="84">
@@ -3819,7 +3819,7 @@
         </is>
       </c>
       <c r="C86" s="33" t="n">
-        <v>75091</v>
+        <v>75692</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3846,7 +3846,7 @@
         <v>5286</v>
       </c>
       <c r="J86" s="202" t="n">
-        <v>0.2592158058678059</v>
+        <v>0.2571593149041637</v>
       </c>
     </row>
     <row r="87">
@@ -3856,7 +3856,7 @@
         </is>
       </c>
       <c r="C87" s="33" t="n">
-        <v>71669</v>
+        <v>71734</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3883,7 +3883,7 @@
         <v>5158</v>
       </c>
       <c r="J87" s="202" t="n">
-        <v>0.225753565334111</v>
+        <v>0.2255496339955474</v>
       </c>
     </row>
     <row r="88">
@@ -3893,7 +3893,7 @@
         </is>
       </c>
       <c r="C88" s="33" t="n">
-        <v>35546</v>
+        <v>35719</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3920,13 +3920,13 @@
         <v>2724</v>
       </c>
       <c r="J88" s="202" t="n">
-        <v>0.3593006245428459</v>
+        <v>0.3575563979238173</v>
       </c>
     </row>
     <row r="90" ht="22" customHeight="1">
       <c r="B90" s="59" t="inlineStr">
         <is>
-          <t>▍ G. 注意股 (資料日 20260706)</t>
+          <t>▍ G. 注意股 (資料日 20260707)</t>
         </is>
       </c>
     </row>
@@ -4330,7 +4330,7 @@
     <row r="112" ht="22" customHeight="1">
       <c r="B112" s="65" t="inlineStr">
         <is>
-          <t>▍ I. 未來 30 天除權息 (有效 270 檔, 已剔除過期)</t>
+          <t>▍ I. 未來 30 天除權息 (有效 260 檔, 已剔除過期)</t>
         </is>
       </c>
     </row>
@@ -4364,17 +4364,17 @@
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260707</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>00946</t>
+          <t>2408</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>群益科技高息成長</t>
+          <t>南亞科</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -4383,23 +4383,23 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>0.058</v>
+        <v>1.347149</v>
       </c>
     </row>
     <row r="115">
       <c r="B115" s="41" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260707</t>
         </is>
       </c>
       <c r="C115" s="41" t="inlineStr">
         <is>
-          <t>00953B</t>
+          <t>2417</t>
         </is>
       </c>
       <c r="D115" s="41" t="inlineStr">
         <is>
-          <t>群益優選非投等債</t>
+          <t>圓剛</t>
         </is>
       </c>
       <c r="E115" s="41" t="inlineStr">
@@ -4408,23 +4408,23 @@
         </is>
       </c>
       <c r="F115" s="41" t="n">
-        <v>0.061</v>
+        <v>0.250119</v>
       </c>
     </row>
     <row r="116">
       <c r="B116" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260707</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>00985B</t>
+          <t>2454</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>群益ESG投等債0-5</t>
+          <t>聯發科</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -4433,23 +4433,23 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>0.048</v>
+        <v>24.500215</v>
       </c>
     </row>
     <row r="117">
       <c r="B117" s="41" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260707</t>
         </is>
       </c>
       <c r="C117" s="41" t="inlineStr">
         <is>
-          <t>00997A</t>
+          <t>2536</t>
         </is>
       </c>
       <c r="D117" s="41" t="inlineStr">
         <is>
-          <t>主動群益美國增長</t>
+          <t>宏普</t>
         </is>
       </c>
       <c r="E117" s="41" t="inlineStr">
@@ -4458,23 +4458,23 @@
         </is>
       </c>
       <c r="F117" s="41" t="n">
-        <v>0.37</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260707</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>1307</t>
+          <t>3048</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>三芳</t>
+          <t>益登</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -4483,23 +4483,23 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>2.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="119">
       <c r="B119" s="41" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260707</t>
         </is>
       </c>
       <c r="C119" s="41" t="inlineStr">
         <is>
-          <t>2373</t>
+          <t>6257</t>
         </is>
       </c>
       <c r="D119" s="41" t="inlineStr">
         <is>
-          <t>震旦行</t>
+          <t>矽格</t>
         </is>
       </c>
       <c r="E119" s="41" t="inlineStr">
@@ -4508,23 +4508,23 @@
         </is>
       </c>
       <c r="F119" s="41" t="n">
-        <v>3.7</v>
+        <v>4.249688</v>
       </c>
     </row>
     <row r="120">
       <c r="B120" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260707</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2474</t>
+          <t>6526</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>可成</t>
+          <t>達發</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -4533,23 +4533,23 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>7.113868</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="121">
       <c r="B121" s="41" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260707</t>
         </is>
       </c>
       <c r="C121" s="41" t="inlineStr">
         <is>
-          <t>2615</t>
+          <t>6591</t>
         </is>
       </c>
       <c r="D121" s="41" t="inlineStr">
         <is>
-          <t>萬海</t>
+          <t>動力-KY</t>
         </is>
       </c>
       <c r="E121" s="41" t="inlineStr">
@@ -4558,23 +4558,23 @@
         </is>
       </c>
       <c r="F121" s="41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="122">
       <c r="B122" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260707</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2904</t>
+          <t>6862</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>匯僑</t>
+          <t>三集瑞-KY</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -4583,23 +4583,23 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>0.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123">
       <c r="B123" s="41" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260707</t>
         </is>
       </c>
       <c r="C123" s="41" t="inlineStr">
         <is>
-          <t>3037</t>
+          <t>9945</t>
         </is>
       </c>
       <c r="D123" s="41" t="inlineStr">
         <is>
-          <t>欣興</t>
+          <t>潤泰新</t>
         </is>
       </c>
       <c r="E123" s="41" t="inlineStr">
@@ -4608,48 +4608,48 @@
         </is>
       </c>
       <c r="F123" s="41" t="n">
-        <v>1.980153</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="124">
       <c r="B124" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260708</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>3557</t>
+          <t>1229</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>嘉威</t>
+          <t>聯華</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>息</t>
+          <t>權息</t>
         </is>
       </c>
       <c r="F124" t="n">
-        <v>0.3</v>
+        <v>1.801172</v>
       </c>
     </row>
     <row r="125">
       <c r="B125" s="41" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260708</t>
         </is>
       </c>
       <c r="C125" s="41" t="inlineStr">
         <is>
-          <t>3704</t>
+          <t>1303</t>
         </is>
       </c>
       <c r="D125" s="41" t="inlineStr">
         <is>
-          <t>合勤控</t>
+          <t>南亞</t>
         </is>
       </c>
       <c r="E125" s="41" t="inlineStr">
@@ -4658,23 +4658,23 @@
         </is>
       </c>
       <c r="F125" s="41" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="126">
       <c r="B126" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260708</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>5538</t>
+          <t>2028</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>東明-KY</t>
+          <t>威致</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -4683,23 +4683,23 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>1.5</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="127">
       <c r="B127" s="41" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260708</t>
         </is>
       </c>
       <c r="C127" s="41" t="inlineStr">
         <is>
-          <t>6155</t>
+          <t>2049</t>
         </is>
       </c>
       <c r="D127" s="41" t="inlineStr">
         <is>
-          <t>鈞寶</t>
+          <t>上銀</t>
         </is>
       </c>
       <c r="E127" s="41" t="inlineStr">
@@ -4708,23 +4708,23 @@
         </is>
       </c>
       <c r="F127" s="41" t="n">
-        <v>0.8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="128">
       <c r="B128" t="inlineStr">
         <is>
-          <t>20260706</t>
+          <t>20260708</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>6754</t>
+          <t>2303</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>匯僑設計</t>
+          <t>聯電</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -4733,7 +4733,7 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>3.5</v>
+        <v>2.608082</v>
       </c>
     </row>
   </sheetData>
@@ -5034,9 +5034,9 @@
       </c>
     </row>
     <row r="30">
-      <c r="C30" s="69" t="inlineStr">
-        <is>
-          <t>除權息 22 檔 (00946 / 00953B / 00985B ...)</t>
+      <c r="C30" s="71" t="inlineStr">
+        <is>
+          <t>今日無除權息</t>
         </is>
       </c>
     </row>
@@ -11090,7 +11090,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="B3" s="98" t="inlineStr">
         <is>
-          <t>大牌分析師 近 53/53 交易日出手 2561 次 (532 檔), 風格分布: 隔日沖近似 39% / 當沖 13% / 留倉 48%, 漲停命中 4% (其中 🔒鎖漲停 4%), 前 5 大集中 24%, 長線部位 62% (38 檔), ⚠️ 處置股部位 12% (36 檔), 📦 連續囤貨 29 檔 (最長 13 天 009816, 皆已停止)。 主軸: 高頻交易/持續進場/📦 連續囤貨。</t>
+          <t>大牌分析師 近 53/53 交易日出手 2561 次 (532 檔), 風格分布: 隔日沖近似 39% / 當沖 13% / 留倉 48%, 漲停命中 4% (其中 🔒鎖漲停 4%), 前 5 大集中 24%, 長線部位 62% (38 檔), ⚠️ 處置股部位 11% (34 檔), 📦 連續囤貨 29 檔 (最長 13 天 009816, 皆已停止)。 主軸: 高頻交易/持續進場/📦 連續囤貨。</t>
         </is>
       </c>
     </row>
@@ -27267,31 +27267,31 @@
       <c r="C416" s="178" t="n"/>
       <c r="D416" s="175" t="inlineStr">
         <is>
-          <t>聯傑(3094)</t>
+          <t>菱生(2369)</t>
         </is>
       </c>
       <c r="E416" s="176" t="n">
-        <v>1475</v>
+        <v>1893</v>
       </c>
       <c r="F416" s="176" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="G416" s="176" t="n">
-        <v>6328</v>
+        <v>8177</v>
       </c>
       <c r="H416" s="176" t="n">
-        <v>4</v>
+        <v>115</v>
       </c>
       <c r="I416" s="176" t="n">
-        <v>6324</v>
+        <v>8062</v>
       </c>
       <c r="J416" s="177" t="n">
-        <v>42.9</v>
+        <v>43.2</v>
       </c>
       <c r="K416" s="177" t="n">
-        <v>43</v>
-      </c>
-      <c r="L416" s="220">
+        <v>42.74</v>
+      </c>
+      <c r="L416" s="219">
         <f>F416*(K416-J416)</f>
         <v/>
       </c>
@@ -27302,29 +27302,29 @@
       <c r="C417" s="178" t="n"/>
       <c r="D417" s="175" t="inlineStr">
         <is>
-          <t>大亞(1609)</t>
+          <t>聯傑(3094)</t>
         </is>
       </c>
       <c r="E417" s="176" t="n">
-        <v>1012</v>
+        <v>1475</v>
       </c>
       <c r="F417" s="176" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G417" s="176" t="n">
-        <v>4427</v>
+        <v>6328</v>
       </c>
       <c r="H417" s="176" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="I417" s="176" t="n">
-        <v>4395</v>
+        <v>6324</v>
       </c>
       <c r="J417" s="177" t="n">
-        <v>43.75</v>
+        <v>42.9</v>
       </c>
       <c r="K417" s="177" t="n">
-        <v>45.86</v>
+        <v>43</v>
       </c>
       <c r="L417" s="220">
         <f>F417*(K417-J417)</f>
@@ -27337,31 +27337,31 @@
       <c r="C418" s="178" t="n"/>
       <c r="D418" s="175" t="inlineStr">
         <is>
-          <t>長榮航太(2645)</t>
+          <t>大亞(1609)</t>
         </is>
       </c>
       <c r="E418" s="176" t="n">
-        <v>63</v>
+        <v>1012</v>
       </c>
       <c r="F418" s="176" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="G418" s="176" t="n">
-        <v>1489</v>
+        <v>4427</v>
       </c>
       <c r="H418" s="176" t="n">
-        <v>635</v>
+        <v>32</v>
       </c>
       <c r="I418" s="176" t="n">
-        <v>854</v>
+        <v>4395</v>
       </c>
       <c r="J418" s="177" t="n">
-        <v>236.33</v>
+        <v>43.75</v>
       </c>
       <c r="K418" s="177" t="n">
-        <v>235.3</v>
-      </c>
-      <c r="L418" s="219">
+        <v>45.86</v>
+      </c>
+      <c r="L418" s="220">
         <f>F418*(K418-J418)</f>
         <v/>
       </c>
@@ -27613,29 +27613,29 @@
       <c r="C425" s="178" t="n"/>
       <c r="D425" s="175" t="inlineStr">
         <is>
-          <t>廣閎科(6693)</t>
+          <t>映泰(2399)</t>
         </is>
       </c>
       <c r="E425" s="176" t="n">
-        <v>30</v>
+        <v>158</v>
       </c>
       <c r="F425" s="176" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="G425" s="176" t="n">
-        <v>836</v>
+        <v>869</v>
       </c>
       <c r="H425" s="176" t="n">
-        <v>0</v>
+        <v>148</v>
       </c>
       <c r="I425" s="176" t="n">
-        <v>836</v>
+        <v>721</v>
       </c>
       <c r="J425" s="177" t="n">
-        <v>278.8</v>
+        <v>55</v>
       </c>
       <c r="K425" s="177" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="L425" s="220">
         <f>F425*(K425-J425)</f>
@@ -27646,25 +27646,46 @@
       <c r="A426" s="178" t="n"/>
       <c r="B426" s="178" t="n"/>
       <c r="C426" s="178" t="n"/>
-      <c r="D426" s="180" t="inlineStr">
-        <is>
-          <t>⚪ 今日漲停僅 6 檔</t>
-        </is>
-      </c>
-      <c r="E426" s="176" t="n"/>
-      <c r="F426" s="176" t="n"/>
-      <c r="G426" s="176" t="n"/>
-      <c r="H426" s="176" t="n"/>
-      <c r="I426" s="176" t="n"/>
-      <c r="J426" s="177" t="n"/>
-      <c r="K426" s="177" t="n"/>
-      <c r="L426" s="221" t="n"/>
+      <c r="D426" s="175" t="inlineStr">
+        <is>
+          <t>廣閎科(6693)</t>
+        </is>
+      </c>
+      <c r="E426" s="176" t="n">
+        <v>30</v>
+      </c>
+      <c r="F426" s="176" t="n">
+        <v>0</v>
+      </c>
+      <c r="G426" s="176" t="n">
+        <v>836</v>
+      </c>
+      <c r="H426" s="176" t="n">
+        <v>0</v>
+      </c>
+      <c r="I426" s="176" t="n">
+        <v>836</v>
+      </c>
+      <c r="J426" s="177" t="n">
+        <v>278.8</v>
+      </c>
+      <c r="K426" s="177" t="n">
+        <v>0</v>
+      </c>
+      <c r="L426" s="220">
+        <f>F426*(K426-J426)</f>
+        <v/>
+      </c>
     </row>
     <row r="427" ht="16.5" customHeight="1">
       <c r="A427" s="178" t="n"/>
       <c r="B427" s="178" t="n"/>
       <c r="C427" s="178" t="n"/>
-      <c r="D427" s="175" t="n"/>
+      <c r="D427" s="180" t="inlineStr">
+        <is>
+          <t>⚪ 今日漲停僅 7 檔</t>
+        </is>
+      </c>
       <c r="E427" s="176" t="n"/>
       <c r="F427" s="176" t="n"/>
       <c r="G427" s="176" t="n"/>

</xml_diff>